<commit_message>
OCA-310 Updated docs according to new requirements
</commit_message>
<xml_diff>
--- a/backend/docs/_Occacia - Planning.xlsx
+++ b/backend/docs/_Occacia - Planning.xlsx
@@ -16,10 +16,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={babbecaf-4c3f-4f4e-b310-f9be7b047401}</author>
+    <author>tc={f4052b6d-55af-4393-a443-57f57dc5c9a9}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{babbecaf-4c3f-4f4e-b310-f9be7b047401}" ref="I10">
+    <comment authorId="0" xr:uid="{f4052b6d-55af-4393-a443-57f57dc5c9a9}" ref="I10">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1219" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1315" uniqueCount="494">
   <si>
     <t>UC ID</t>
   </si>
@@ -2383,18 +2383,9 @@
     <r>
       <rPr>
         <rFont val="Arial"/>
-        <b/>
         <color theme="1"/>
       </rPr>
-      <t>Part A — Create Event</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">
-1. Customer taps Create Event.
+      <t xml:space="preserve">1. Customer taps Create Event.
 2. System displays an event creation form.
 3. System shows Event Type dropdown with examples (e.g., </t>
     </r>
@@ -2607,7 +2598,7 @@
     <t>UC-13</t>
   </si>
   <si>
-    <t>Interact with Event Chat</t>
+    <t>Interact with Event Chat (Scheduling + Recurrence + Reminders)</t>
   </si>
   <si>
     <t>AI Recommendation Engine</t>
@@ -2648,21 +2639,27 @@
         <rFont val="Arial"/>
         <color theme="1"/>
       </rPr>
-      <t xml:space="preserve"> Event exists.</t>
+      <t xml:space="preserve"> Event exists. Notification permission is available (system can request it). If external calendar sync is used, the customer has connected a calendar provider (or system will prompt to connect).</t>
     </r>
   </si>
   <si>
     <t>1. Customer opens the Event Chat for a selected event (either immediately after creating an event or from the Events List).
 2. System displays the Event Chat interface.
 3. If tasks are missing/incomplete, system shows template-based suggested tasks based on Event Type.
-4. System asks lightweight planning prompts to complete key details (e.g., When is it? Where is it? What do you need? Budget?), using Persona preferences when available.
+4. System asks lightweight planning prompts to complete key details (e.g., Schedule: When is it? One-time or recurring? Time zone? All-day or timed? Recurrence frequency and end? Reminder offsets (e.g., 7 days before / 1 day before / same day)? Where is it? What do you need? Budget?), using Persona preferences when available.
 5. Customer provides additional information through chat (requirements, constraints, preferences).
-6. System analyzes customer messages, identifies missing/unclear details, and asks follow-up questions as needed.
-7. System generates or refines a list of proposed tasks (editable) and a summarized event context.
-8. Customer reviews and adjusts tasks (edit/add/remove; optionally mark “Needs vendor” + category).
-9. Customer taps Confirm Tasks.
-10. System saves confirmed tasks and updates the Event status to Active (if it was Draft).
-11. System prompts the customer to proceed to recommendation generation.</t>
+6. System validates schedule inputs (date/time format, time zone, recurrence rule, reminder offsets) and asks follow-up questions if ambiguous (e.g., ‘Every year on this date?’ for birthdays).
+7. System offers calendar behavior options:
+     - Local reminders only (in-app/push/email), OR
+     - Sync to external calendar (Google/Apple/Microsoft) if connected.
+8. If external sync is chosen and not connected, system prompts customer to connect a calendar provider (OAuth) and then resumes the chat.
+9. System generates or refines a list of proposed tasks (editable) and a summarized event context including the saved schedule, recurrence pattern, next occurrence, and reminder plan.
+10. Customer reviews and adjusts tasks (edit/add/remove; optionally mark “Needs vendor” + category).
+11. Customer taps Confirm Tasks.
+12. System saves confirmed tasks and schedule settings (date/time/timezone/recurrence/reminders) and updates the Event status to Active (if it was Draft).
+If reminders are enabled, system schedules notifications.
+If external calendar sync is enabled, system creates/updates the external calendar event/series.
+13. System prompts the customer to proceed to recommendation generation and shows confirmation of schedule/reminders (and calendar link if synced).</t>
   </si>
   <si>
     <r>
@@ -2679,7 +2676,7 @@
         <rFont val="Arial"/>
         <color theme="1"/>
       </rPr>
-      <t xml:space="preserve">Customer exits chat without Confirm Tasks → Event remains </t>
+      <t xml:space="preserve">1. Customer exits chat without Confirm Tasks → Event remains </t>
     </r>
     <r>
       <rPr>
@@ -2710,9 +2707,14 @@
         <color theme="1"/>
       </rPr>
       <t xml:space="preserve">
-AI/task generation fails → system shows template tasks and allows manual task creation; customer can still confirm tasks.
-Customer confirms with zero tasks:
+2. AI/task generation fails → system shows template tasks and allows manual task creation; customer can still confirm tasks.
+3. Customer confirms with zero tasks:
      - block with message “Add at least 1 task”
+4. Customer sets “date TBD” / unknown schedule → Event can remain Draft or Active, but recurrence/reminders are not scheduled until a valid date/time is provided.
+5. Customer selects recurring but provides invalid/ambiguous recurrence → System asks clarification (e.g., yearly vs monthly; end date; occurrences limit).
+6. Customer declines notification permission → Event schedule can still be saved, but reminders are disabled (system shows “Enable notifications to get reminders”).
+7. External calendar not connected → System offers “Connect calendar now” or “Skip (local reminders only)”.
+8. External calendar sync fails → Event + tasks still saved; system falls back to local reminders and shows “Calendar sync failed, try again later”.
 </t>
     </r>
     <r>
@@ -2730,9 +2732,11 @@
         <color theme="1"/>
       </rPr>
       <t xml:space="preserve">
-Event context is updated with refined details.
+Event context is updated with refined details including schedule + recurrence + reminder settings.
 A confirmed set of tasks is saved for the event.
 Event is Active and ready for recommendation generation.
+If reminders enabled: reminders are scheduled.
+If calendar sync enabled: external calendar event/series is created/updated.
 </t>
     </r>
     <r>
@@ -2750,8 +2754,8 @@
         <color theme="1"/>
       </rPr>
       <t xml:space="preserve">
-Event remains in its previous state (Draft/Active).
-No changes are saved unless the customer confirms tasks; refinement may be incomplete.</t>
+1. Event remains in its previous state (Draft/Active).
+2. No changes are saved unless the customer confirms tasks; refinement may be incomplete.</t>
     </r>
   </si>
   <si>
@@ -2814,13 +2818,22 @@
 POST /api/v1/customers/events/{eventId}/tasks/confirm (recommended new endpoint; change event status: draft → active )
 PUT /api/v1/customers/events/{eventId}/tasks/{taskId}
 DELETE /api/v1/customers/events/{eventId}/tasks/{taskId}
- </t>
+// Calendar Integration
+PUT /api/v1/customers/events/{eventId}/schedule 
+body includes: startAt, endAt (optional), timezone, isAllDay, recurrenceRule (RRULE or simplified), recurrenceEnd (optional)
+PUT /api/v1/customers/events/{eventId}/reminders
+body includes reminder offsets + channels (push/email/in-app)
+GET /api/v1/customers/calendar/providers
+POST /api/v1/customers/calendar/connect (OAuth start)
+GET /api/v1/customers/calendar/status
+DELETE /api/v1/customers/calendar/disconnect
+PUT /api/v1/customers/events/{eventId}/calendar-sync (enable/disable + provider calendarId)</t>
     </r>
   </si>
   <si>
     <r>
       <rPr/>
-      <t>1. Customer opens the Events List. (</t>
+      <t>1.Customer opens the Events List. (</t>
     </r>
     <r>
       <rPr>
@@ -2833,7 +2846,8 @@
       <rPr/>
       <t>)
 2. Customer selects an event (or is redirected here right after creating one).
-3. System displays the Chat Interface for the selected event. (</t>
+3. System displays the Chat Interface for the selected event.
+(</t>
     </r>
     <r>
       <rPr>
@@ -2845,12 +2859,22 @@
     <r>
       <rPr/>
       <t>)
-4. System shows suggested tasks (from templates) and asks lightweight prompts (When/Where/What needed, etc.).
-5. Customer describes additional requirements or clarifies preferences.
-6. Chat assistant asks follow-up questions and refines the proposed task list.
-7. System shows a summarized view of the refined event and proposed tasks, allowing edits.
-8. Customer taps Confirm Tasks.
-9. System saves tasks, updates Event status (Draft → Active if applicable), and navigates to recommendations. (</t>
+4. System shows suggested tasks (from templates) and prompts for key planning details including scheduling:
+5. When is it? (date/time, timezone, all-day vs timed)
+6. One-time or recurring? (e.g., yearly for birthdays)
+7. Reminder preferences (e.g., 7 days before / 1 day before / same day)
+8. (Optional) Sync to external calendar (Google/Apple/Microsoft)
+9. Customer sets/updates the schedule (one-time or recurring) and selects reminder options.
+10. If reminders are enabled, system requests notification permission (if not already granted).
+If external calendar sync is selected and not connected, system prompts customer to connect a calendar provider (OAuth) and returns to chat on success.
+11. Customer describes additional requirements or clarifies preferences through chat.
+12. Chat assistant asks follow-up questions and refines both the event context (including schedule/recurrence/reminders) and the proposed task list.
+13. System shows a summarized view of the refined event (including next occurrence + reminder plan) and proposed tasks, allowing edits.
+14. Customer taps Confirm Tasks (or Confirm &amp; Activate).
+15. System saves tasks + schedule settings (date/time/timezone/recurrence/reminders), 
+updates Event status (Draft → Active if applicable), schedules reminders, and performs calendar sync if enabled.
+16. System navigates to recommendations.
+(</t>
     </r>
     <r>
       <rPr>
@@ -6346,6 +6370,39 @@
     <t>Set personas linked to an event (replace EVENT_PERSONA links)</t>
   </si>
   <si>
+    <t>/api/v1/customers/events/{eventId}/schedule</t>
+  </si>
+  <si>
+    <t>Get event schedule details (start/end, timezone, all-day) + recurrence rule + next occurrence (if recurring)</t>
+  </si>
+  <si>
+    <t>Upsert event schedule: startAt/endAt/isAllDay/timezone + recurrenceRule (optional) + recurrenceEnd (optional); returns computed nextOccurrence</t>
+  </si>
+  <si>
+    <t>/api/v1/customers/events/{eventId}/reminders</t>
+  </si>
+  <si>
+    <t>Get reminder configuration for the event (offsets + channels + enabled/disabled)</t>
+  </si>
+  <si>
+    <t>Upsert reminders for event: offsets (e.g., 7d/1d/0d) + channels (push/email/in-app); schedules notifications when enabled</t>
+  </si>
+  <si>
+    <t>/api/v1/customers/events/{eventId}/occurrences</t>
+  </si>
+  <si>
+    <t>List upcoming occurrences for recurring events (supports query: from, limit); used to show next dates &amp; reminder preview</t>
+  </si>
+  <si>
+    <t>/api/v1/customers/events/{eventId}/calendar-sync</t>
+  </si>
+  <si>
+    <t>Get per-event calendar sync state (enabled, provider, calendarId, externalEventId, lastSyncAt, lastSyncStatus)</t>
+  </si>
+  <si>
+    <t>Enable/disable per-event sync; select calendarId; create/update external calendar event/series; store externalEventId</t>
+  </si>
+  <si>
     <t>customers/chat</t>
   </si>
   <si>
@@ -6451,7 +6508,20 @@
     <t>/api/v1/customers/events/{eventId}/package-orders</t>
   </si>
   <si>
-    <t>List package orders for an event (tracking screen context)</t>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">List package orders for an event </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FFFF0000"/>
+      </rPr>
+      <t>(tracking screen context)</t>
+    </r>
   </si>
   <si>
     <t>/api/v1/customers/package-orders</t>
@@ -6464,6 +6534,39 @@
   </si>
   <si>
     <t>OPTIONAL: If customer has Package Orders page, get one package order detail (totals, per-task selections, status)</t>
+  </si>
+  <si>
+    <t>customers/calendar</t>
+  </si>
+  <si>
+    <t>/api/v1/customers/calendar/providers</t>
+  </si>
+  <si>
+    <t>List supported external calendar providers (e.g., Google/Microsoft) + capabilities (recurrence supported, scopes)</t>
+  </si>
+  <si>
+    <t>/api/v1/customers/calendar/connect</t>
+  </si>
+  <si>
+    <t>Start calendar OAuth connect; returns authorizationUrl + state (PKCE supported)</t>
+  </si>
+  <si>
+    <t>/api/v1/customers/calendar/exchange-code</t>
+  </si>
+  <si>
+    <t>Exchange OAuth code for tokens and link provider to customer; stores refresh token securely</t>
+  </si>
+  <si>
+    <t>/api/v1/customers/calendar/status</t>
+  </si>
+  <si>
+    <t>Get calendar connection status (connected provider, defaultCalendarId, connectedAt, lastSyncAt)</t>
+  </si>
+  <si>
+    <t>/api/v1/customers/calendar/disconnect</t>
+  </si>
+  <si>
+    <t>Disconnect calendar provider; revoke tokens; stop future sync operations</t>
   </si>
   <si>
     <t>vendors/offerings</t>
@@ -6836,7 +6939,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -7003,11 +7106,14 @@
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -7096,22 +7202,22 @@
 
 <file path=xl/documenttasks/documenttask1.xml><?xml version="1.0" encoding="utf-8"?>
 <Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks">
-  <Task id="{3a44c144-e33a-4aa5-9c23-efabd97bb5e4}">
+  <Task id="{6f6eb6c1-ead3-48aa-b1c0-3409a6d492de}">
     <Anchor>
-      <Comment id="{babbecaf-4c3f-4f4e-b310-f9be7b047401}"/>
+      <Comment id="{f4052b6d-55af-4393-a443-57f57dc5c9a9}"/>
     </Anchor>
     <History>
-      <Event time="2026-01-28T17:56:52.00" id="{ff15648f-b4e2-4f4a-84d0-3b1e04aa49c1}">
+      <Event time="2026-01-28T17:56:52.00" id="{936fa431-8a00-47c6-b7de-ab6f18824e19}">
         <Attribution userId="placeholder@email.com" userName="Dilruk Jayasinghe" userProvider="google-sheets"/>
         <Anchor>
-          <Comment id="{babbecaf-4c3f-4f4e-b310-f9be7b047401}"/>
+          <Comment id="{f4052b6d-55af-4393-a443-57f57dc5c9a9}"/>
         </Anchor>
         <Create/>
       </Event>
-      <Event time="2026-01-28T17:56:52.00" id="{4c9732f8-df74-48fb-867b-e357377454ff}">
+      <Event time="2026-01-28T17:56:52.00" id="{5cb8778b-2cd1-4124-8c4d-1f979c61d0fb}">
         <Attribution userId="placeholder@email.com" userName="Dilruk Jayasinghe" userProvider="google-sheets"/>
         <Anchor>
-          <Comment id="{babbecaf-4c3f-4f4e-b310-f9be7b047401}"/>
+          <Comment id="{f4052b6d-55af-4393-a443-57f57dc5c9a9}"/>
         </Anchor>
         <Assign userId="dilruk.20234022@iit.ac.lk" userName="dilruk.20234022@iit.ac.lk" userProvider="google-sheets"/>
       </Event>
@@ -7130,14 +7236,14 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Dilruk Jayasinghe" id="{381bc60f-7201-49f3-8d31-a5865eb6b4d4}" providerId="google-sheets"/>
-  <x18tc:person displayName="indura.20223174@iit.ac.lk" id="{f8e8e800-a102-4e46-afef-2184d5f69428}" userId="indura.20223174@iit.ac.lk" providerId="google-sheets"/>
-  <x18tc:person displayName="tisal.20221672@iit.ac.lk" id="{ffd29a11-9bc3-4ca0-b8dc-c8536b347263}" userId="tisal.20221672@iit.ac.lk" providerId="google-sheets"/>
-  <x18tc:person displayName="tharindu.20234071@iit.ac.lk" id="{9eb11af5-aecf-4fd7-bf22-7b65ce0401e0}" userId="tharindu.20234071@iit.ac.lk" providerId="google-sheets"/>
-  <x18tc:person displayName="rinusha.20234008@iit.ac.lk" id="{61703c37-ac31-4adc-bf32-6a63379c19ad}" userId="rinusha.20234008@iit.ac.lk" providerId="google-sheets"/>
-  <x18tc:person displayName="pinsara.20221670@iit.ac.lk" id="{5b476da8-499b-4eaf-ab95-60590601842e}" userId="pinsara.20221670@iit.ac.lk" providerId="google-sheets"/>
-  <x18tc:person displayName="himasha.20234048@iit.ac.lk" id="{0de1549d-601d-4cb3-b17e-82ec83485db2}" userId="himasha.20234048@iit.ac.lk" providerId="google-sheets"/>
-  <x18tc:person displayName="dilruk.20234022@iit.ac.lk" id="{6cf36f37-5094-4649-9c8a-ae6547d52ec7}" userId="dilruk.20234022@iit.ac.lk" providerId="google-sheets"/>
+  <x18tc:person displayName="Dilruk Jayasinghe" id="{177d18b9-6f5f-40ed-bfca-b0ce257a299b}" providerId="google-sheets"/>
+  <x18tc:person displayName="indura.20223174@iit.ac.lk" id="{9f09c695-4136-4f78-a02d-f3c34ddc2dcd}" userId="indura.20223174@iit.ac.lk" providerId="google-sheets"/>
+  <x18tc:person displayName="tisal.20221672@iit.ac.lk" id="{c05948fa-d282-41f5-81b2-530f9640c553}" userId="tisal.20221672@iit.ac.lk" providerId="google-sheets"/>
+  <x18tc:person displayName="tharindu.20234071@iit.ac.lk" id="{d663162d-6572-4f41-afb6-e8eade3a21a6}" userId="tharindu.20234071@iit.ac.lk" providerId="google-sheets"/>
+  <x18tc:person displayName="rinusha.20234008@iit.ac.lk" id="{c2f485bf-0822-4ade-839e-58a65fb6f545}" userId="rinusha.20234008@iit.ac.lk" providerId="google-sheets"/>
+  <x18tc:person displayName="pinsara.20221670@iit.ac.lk" id="{31ffb3ce-3cd0-4ac3-aa2d-992fd3f71af5}" userId="pinsara.20221670@iit.ac.lk" providerId="google-sheets"/>
+  <x18tc:person displayName="himasha.20234048@iit.ac.lk" id="{dbcae488-a941-43d9-84a2-d33d89c5ec81}" userId="himasha.20234048@iit.ac.lk" providerId="google-sheets"/>
+  <x18tc:person displayName="dilruk.20234022@iit.ac.lk" id="{68af3b6a-c8a1-4229-8d95-c286b95e4a21}" userId="dilruk.20234022@iit.ac.lk" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -7165,7 +7271,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H123" displayName="Table2" name="Table2" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H137" displayName="Table2" name="Table2" id="2">
   <tableColumns count="8">
     <tableColumn name="Type" id="1"/>
     <tableColumn name="Resource" id="2"/>
@@ -7376,20 +7482,20 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="I10" dT="2026-01-28T17:56:52.00" personId="{381bc60f-7201-49f3-8d31-a5865eb6b4d4}" id="{babbecaf-4c3f-4f4e-b310-f9be7b047401}" done="1">
+  <x18tc:threadedComment ref="I10" dT="2026-01-28T17:56:52.00" personId="{177d18b9-6f5f-40ed-bfca-b0ce257a299b}" id="{f4052b6d-55af-4393-a443-57f57dc5c9a9}" done="1">
     <x18tc:text xml:space="preserve">TODO: Change Plan -&gt; Event and Event -&gt; Task
 cc: @pinsara.20221670@iit.ac.lk @tisal.20221672@iit.ac.lk @rinusha.20234008@iit.ac.lk @himasha.20234048@iit.ac.lk @indura.20223174@iit.ac.lk 
 @dilruk.20234022@iit.ac.lk 
 @tharindu.20234071@iit.ac.lk
 Assigned to dilruk.20234022@iit.ac.lk</x18tc:text>
     <x18tc:mentions>
-      <x18tc:mention mentionpersonId="{5b476da8-499b-4eaf-ab95-60590601842e}" mentionId="{19be491e-73f7-4f8c-bcd5-3527ee788c10}" startIndex="50" length="27"/>
-      <x18tc:mention mentionpersonId="{ffd29a11-9bc3-4ca0-b8dc-c8536b347263}" mentionId="{eb512a8f-1e6c-46fb-a846-74ee45d351d4}" startIndex="78" length="25"/>
-      <x18tc:mention mentionpersonId="{61703c37-ac31-4adc-bf32-6a63379c19ad}" mentionId="{9c04573a-5d7e-42c2-840d-8169868fc85e}" startIndex="104" length="27"/>
-      <x18tc:mention mentionpersonId="{0de1549d-601d-4cb3-b17e-82ec83485db2}" mentionId="{798063ec-cca3-4f5e-8d93-e06d62f19e84}" startIndex="132" length="27"/>
-      <x18tc:mention mentionpersonId="{f8e8e800-a102-4e46-afef-2184d5f69428}" mentionId="{5c73d72e-f1bf-4f39-8992-2a06e8b023bb}" startIndex="160" length="26"/>
-      <x18tc:mention mentionpersonId="{6cf36f37-5094-4649-9c8a-ae6547d52ec7}" mentionId="{51c04b53-a1f4-4f3a-9639-77e64c15cf8b}" startIndex="188" length="26"/>
-      <x18tc:mention mentionpersonId="{9eb11af5-aecf-4fd7-bf22-7b65ce0401e0}" mentionId="{aa64ae1d-30de-4417-84f1-b7302cad4511}" startIndex="216" length="28"/>
+      <x18tc:mention mentionpersonId="{31ffb3ce-3cd0-4ac3-aa2d-992fd3f71af5}" mentionId="{fcbf38fd-f25f-4f88-9cbe-257c800aa8f3}" startIndex="50" length="27"/>
+      <x18tc:mention mentionpersonId="{c05948fa-d282-41f5-81b2-530f9640c553}" mentionId="{e2a90007-e3fc-473d-b94a-10f2c6caaa80}" startIndex="78" length="25"/>
+      <x18tc:mention mentionpersonId="{c2f485bf-0822-4ade-839e-58a65fb6f545}" mentionId="{d104e776-7db6-4d2e-b579-6f0eff1012c8}" startIndex="104" length="27"/>
+      <x18tc:mention mentionpersonId="{dbcae488-a941-43d9-84a2-d33d89c5ec81}" mentionId="{ae840b97-445c-488b-919f-05215868740b}" startIndex="132" length="27"/>
+      <x18tc:mention mentionpersonId="{9f09c695-4136-4f78-a02d-f3c34ddc2dcd}" mentionId="{95f4e4ab-66cf-4633-a92a-a62a8a4eaae5}" startIndex="160" length="26"/>
+      <x18tc:mention mentionpersonId="{68af3b6a-c8a1-4229-8d95-c286b95e4a21}" mentionId="{b036dcd3-11ae-43f6-be8c-e4ad96a5997a}" startIndex="188" length="26"/>
+      <x18tc:mention mentionpersonId="{d663162d-6572-4f41-afb6-e8eade3a21a6}" mentionId="{819dda43-93a3-4993-8d7f-52bba72610bc}" startIndex="216" length="28"/>
     </x18tc:mentions>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -7410,7 +7516,7 @@
     <col customWidth="1" min="6" max="6" width="74.63"/>
     <col customWidth="1" min="7" max="7" width="66.5"/>
     <col customWidth="1" min="8" max="8" width="14.25"/>
-    <col customWidth="1" min="9" max="9" width="87.5"/>
+    <col customWidth="1" min="9" max="9" width="95.38"/>
     <col customWidth="1" min="10" max="10" width="89.38"/>
     <col customWidth="1" min="12" max="12" width="15.38"/>
     <col customWidth="1" min="13" max="13" width="15.5"/>
@@ -8209,7 +8315,7 @@
       <c r="AD13" s="4"/>
       <c r="AE13" s="4"/>
     </row>
-    <row r="14" ht="436.5" customHeight="1">
+    <row r="14" ht="694.5" customHeight="1">
       <c r="A14" s="5" t="s">
         <v>116</v>
       </c>
@@ -44079,14 +44185,30 @@
       <c r="AA50" s="4"/>
     </row>
     <row r="51" ht="22.5" customHeight="1">
-      <c r="A51" s="55"/>
-      <c r="B51" s="47"/>
-      <c r="C51" s="48"/>
-      <c r="D51" s="48"/>
-      <c r="E51" s="49"/>
-      <c r="F51" s="50"/>
-      <c r="G51" s="49"/>
-      <c r="H51" s="49"/>
+      <c r="A51" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B51" s="47" t="s">
+        <v>339</v>
+      </c>
+      <c r="C51" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D51" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E51" s="49" t="s">
+        <v>348</v>
+      </c>
+      <c r="F51" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="G51" s="49" t="s">
+        <v>116</v>
+      </c>
+      <c r="H51" s="49" t="s">
+        <v>349</v>
+      </c>
       <c r="I51" s="4"/>
       <c r="J51" s="4"/>
       <c r="K51" s="4"/>
@@ -44112,24 +44234,24 @@
         <v>16</v>
       </c>
       <c r="B52" s="47" t="s">
+        <v>339</v>
+      </c>
+      <c r="C52" s="56" t="s">
+        <v>309</v>
+      </c>
+      <c r="D52" s="56" t="s">
+        <v>310</v>
+      </c>
+      <c r="E52" s="57" t="s">
         <v>348</v>
       </c>
-      <c r="C52" s="48" t="s">
-        <v>261</v>
-      </c>
-      <c r="D52" s="48" t="s">
-        <v>258</v>
-      </c>
-      <c r="E52" s="49" t="s">
-        <v>349</v>
-      </c>
-      <c r="F52" s="48" t="s">
+      <c r="F52" s="56" t="s">
         <v>26</v>
       </c>
-      <c r="G52" s="49" t="s">
+      <c r="G52" s="57" t="s">
         <v>116</v>
       </c>
-      <c r="H52" s="49" t="s">
+      <c r="H52" s="57" t="s">
         <v>350</v>
       </c>
       <c r="I52" s="4"/>
@@ -44157,24 +44279,24 @@
         <v>16</v>
       </c>
       <c r="B53" s="47" t="s">
-        <v>348</v>
-      </c>
-      <c r="C53" s="48" t="s">
-        <v>261</v>
-      </c>
-      <c r="D53" s="48" t="s">
-        <v>258</v>
-      </c>
-      <c r="E53" s="49" t="s">
+        <v>339</v>
+      </c>
+      <c r="C53" s="56" t="s">
+        <v>306</v>
+      </c>
+      <c r="D53" s="56" t="s">
+        <v>262</v>
+      </c>
+      <c r="E53" s="57" t="s">
         <v>351</v>
       </c>
-      <c r="F53" s="48" t="s">
+      <c r="F53" s="56" t="s">
         <v>26</v>
       </c>
-      <c r="G53" s="49" t="s">
+      <c r="G53" s="57" t="s">
         <v>116</v>
       </c>
-      <c r="H53" s="49" t="s">
+      <c r="H53" s="57" t="s">
         <v>352</v>
       </c>
       <c r="I53" s="4"/>
@@ -44202,25 +44324,25 @@
         <v>16</v>
       </c>
       <c r="B54" s="47" t="s">
+        <v>339</v>
+      </c>
+      <c r="C54" s="56" t="s">
+        <v>309</v>
+      </c>
+      <c r="D54" s="56" t="s">
+        <v>310</v>
+      </c>
+      <c r="E54" s="57" t="s">
+        <v>351</v>
+      </c>
+      <c r="F54" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="G54" s="57" t="s">
+        <v>116</v>
+      </c>
+      <c r="H54" s="57" t="s">
         <v>353</v>
-      </c>
-      <c r="C54" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="D54" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E54" s="49" t="s">
-        <v>354</v>
-      </c>
-      <c r="F54" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="G54" s="49" t="s">
-        <v>116</v>
-      </c>
-      <c r="H54" s="56" t="s">
-        <v>355</v>
       </c>
       <c r="I54" s="4"/>
       <c r="J54" s="4"/>
@@ -44243,14 +44365,30 @@
       <c r="AA54" s="4"/>
     </row>
     <row r="55" ht="22.5" customHeight="1">
-      <c r="A55" s="55"/>
-      <c r="B55" s="47"/>
-      <c r="C55" s="48"/>
-      <c r="D55" s="48"/>
-      <c r="E55" s="49"/>
-      <c r="F55" s="50"/>
-      <c r="G55" s="49"/>
-      <c r="H55" s="49"/>
+      <c r="A55" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B55" s="47" t="s">
+        <v>339</v>
+      </c>
+      <c r="C55" s="56" t="s">
+        <v>306</v>
+      </c>
+      <c r="D55" s="56" t="s">
+        <v>262</v>
+      </c>
+      <c r="E55" s="57" t="s">
+        <v>354</v>
+      </c>
+      <c r="F55" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="G55" s="57" t="s">
+        <v>116</v>
+      </c>
+      <c r="H55" s="57" t="s">
+        <v>355</v>
+      </c>
       <c r="I55" s="4"/>
       <c r="J55" s="4"/>
       <c r="K55" s="4"/>
@@ -44276,25 +44414,25 @@
         <v>16</v>
       </c>
       <c r="B56" s="47" t="s">
+        <v>339</v>
+      </c>
+      <c r="C56" s="56" t="s">
+        <v>306</v>
+      </c>
+      <c r="D56" s="56" t="s">
+        <v>262</v>
+      </c>
+      <c r="E56" s="57" t="s">
         <v>356</v>
       </c>
-      <c r="C56" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="D56" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E56" s="49" t="s">
+      <c r="F56" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="G56" s="57" t="s">
+        <v>116</v>
+      </c>
+      <c r="H56" s="57" t="s">
         <v>357</v>
-      </c>
-      <c r="F56" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="G56" s="49" t="s">
-        <v>116</v>
-      </c>
-      <c r="H56" s="49" t="s">
-        <v>358</v>
       </c>
       <c r="I56" s="4"/>
       <c r="J56" s="4"/>
@@ -44321,25 +44459,25 @@
         <v>16</v>
       </c>
       <c r="B57" s="47" t="s">
+        <v>339</v>
+      </c>
+      <c r="C57" s="56" t="s">
+        <v>309</v>
+      </c>
+      <c r="D57" s="56" t="s">
+        <v>310</v>
+      </c>
+      <c r="E57" s="57" t="s">
         <v>356</v>
       </c>
-      <c r="C57" s="48" t="s">
-        <v>257</v>
-      </c>
-      <c r="D57" s="48" t="s">
-        <v>258</v>
-      </c>
-      <c r="E57" s="49" t="s">
-        <v>357</v>
-      </c>
-      <c r="F57" s="48" t="s">
+      <c r="F57" s="56" t="s">
         <v>26</v>
       </c>
-      <c r="G57" s="49" t="s">
+      <c r="G57" s="57" t="s">
         <v>116</v>
       </c>
-      <c r="H57" s="49" t="s">
-        <v>359</v>
+      <c r="H57" s="57" t="s">
+        <v>358</v>
       </c>
       <c r="I57" s="4"/>
       <c r="J57" s="4"/>
@@ -44362,30 +44500,14 @@
       <c r="AA57" s="4"/>
     </row>
     <row r="58" ht="22.5" customHeight="1">
-      <c r="A58" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="B58" s="47" t="s">
-        <v>356</v>
-      </c>
-      <c r="C58" s="48" t="s">
-        <v>261</v>
-      </c>
-      <c r="D58" s="48" t="s">
-        <v>258</v>
-      </c>
-      <c r="E58" s="49" t="s">
-        <v>360</v>
-      </c>
-      <c r="F58" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="G58" s="49" t="s">
-        <v>116</v>
-      </c>
-      <c r="H58" s="49" t="s">
-        <v>361</v>
-      </c>
+      <c r="A58" s="55"/>
+      <c r="B58" s="47"/>
+      <c r="C58" s="48"/>
+      <c r="D58" s="48"/>
+      <c r="E58" s="49"/>
+      <c r="F58" s="50"/>
+      <c r="G58" s="49"/>
+      <c r="H58" s="49"/>
       <c r="I58" s="4"/>
       <c r="J58" s="4"/>
       <c r="K58" s="4"/>
@@ -44411,16 +44533,16 @@
         <v>16</v>
       </c>
       <c r="B59" s="47" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="C59" s="48" t="s">
-        <v>309</v>
+        <v>261</v>
       </c>
       <c r="D59" s="48" t="s">
-        <v>310</v>
+        <v>258</v>
       </c>
       <c r="E59" s="49" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="F59" s="48" t="s">
         <v>26</v>
@@ -44429,7 +44551,7 @@
         <v>116</v>
       </c>
       <c r="H59" s="49" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="I59" s="4"/>
       <c r="J59" s="4"/>
@@ -44456,13 +44578,13 @@
         <v>16</v>
       </c>
       <c r="B60" s="47" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="C60" s="48" t="s">
-        <v>336</v>
+        <v>261</v>
       </c>
       <c r="D60" s="48" t="s">
-        <v>337</v>
+        <v>258</v>
       </c>
       <c r="E60" s="49" t="s">
         <v>362</v>
@@ -44474,7 +44596,7 @@
         <v>116</v>
       </c>
       <c r="H60" s="49" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="I60" s="4"/>
       <c r="J60" s="4"/>
@@ -44501,24 +44623,24 @@
         <v>16</v>
       </c>
       <c r="B61" s="47" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="C61" s="48" t="s">
-        <v>261</v>
+        <v>306</v>
       </c>
       <c r="D61" s="48" t="s">
-        <v>258</v>
-      </c>
-      <c r="E61" s="57" t="s">
+        <v>262</v>
+      </c>
+      <c r="E61" s="49" t="s">
         <v>365</v>
       </c>
       <c r="F61" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="G61" s="57" t="s">
-        <v>177</v>
-      </c>
-      <c r="H61" s="57" t="s">
+      <c r="G61" s="49" t="s">
+        <v>116</v>
+      </c>
+      <c r="H61" s="58" t="s">
         <v>366</v>
       </c>
       <c r="I61" s="4"/>
@@ -44578,10 +44700,10 @@
         <v>367</v>
       </c>
       <c r="C63" s="48" t="s">
-        <v>261</v>
+        <v>306</v>
       </c>
       <c r="D63" s="48" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="E63" s="49" t="s">
         <v>368</v>
@@ -44590,7 +44712,7 @@
         <v>26</v>
       </c>
       <c r="G63" s="49" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="H63" s="49" t="s">
         <v>369</v>
@@ -44623,22 +44745,22 @@
         <v>367</v>
       </c>
       <c r="C64" s="48" t="s">
-        <v>306</v>
+        <v>257</v>
       </c>
       <c r="D64" s="48" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="E64" s="49" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="F64" s="48" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="49" t="s">
-        <v>140</v>
+        <v>116</v>
       </c>
       <c r="H64" s="49" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="I64" s="4"/>
       <c r="J64" s="4"/>
@@ -44661,14 +44783,30 @@
       <c r="AA64" s="4"/>
     </row>
     <row r="65" ht="22.5" customHeight="1">
-      <c r="A65" s="55"/>
-      <c r="B65" s="47"/>
-      <c r="C65" s="48"/>
-      <c r="D65" s="48"/>
-      <c r="E65" s="49"/>
-      <c r="F65" s="50"/>
-      <c r="G65" s="49"/>
-      <c r="H65" s="49"/>
+      <c r="A65" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B65" s="47" t="s">
+        <v>367</v>
+      </c>
+      <c r="C65" s="48" t="s">
+        <v>261</v>
+      </c>
+      <c r="D65" s="48" t="s">
+        <v>258</v>
+      </c>
+      <c r="E65" s="49" t="s">
+        <v>371</v>
+      </c>
+      <c r="F65" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="G65" s="49" t="s">
+        <v>116</v>
+      </c>
+      <c r="H65" s="49" t="s">
+        <v>372</v>
+      </c>
       <c r="I65" s="4"/>
       <c r="J65" s="4"/>
       <c r="K65" s="4"/>
@@ -44694,13 +44832,13 @@
         <v>16</v>
       </c>
       <c r="B66" s="47" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="C66" s="48" t="s">
-        <v>257</v>
+        <v>309</v>
       </c>
       <c r="D66" s="48" t="s">
-        <v>258</v>
+        <v>310</v>
       </c>
       <c r="E66" s="49" t="s">
         <v>373</v>
@@ -44709,7 +44847,7 @@
         <v>26</v>
       </c>
       <c r="G66" s="49" t="s">
-        <v>140</v>
+        <v>116</v>
       </c>
       <c r="H66" s="49" t="s">
         <v>374</v>
@@ -44739,13 +44877,13 @@
         <v>16</v>
       </c>
       <c r="B67" s="47" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="C67" s="48" t="s">
-        <v>306</v>
+        <v>336</v>
       </c>
       <c r="D67" s="48" t="s">
-        <v>262</v>
+        <v>337</v>
       </c>
       <c r="E67" s="49" t="s">
         <v>373</v>
@@ -44754,7 +44892,7 @@
         <v>26</v>
       </c>
       <c r="G67" s="49" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="H67" s="49" t="s">
         <v>375</v>
@@ -44784,13 +44922,13 @@
         <v>16</v>
       </c>
       <c r="B68" s="47" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="C68" s="48" t="s">
-        <v>306</v>
+        <v>261</v>
       </c>
       <c r="D68" s="48" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="E68" s="49" t="s">
         <v>376</v>
@@ -44799,7 +44937,7 @@
         <v>26</v>
       </c>
       <c r="G68" s="49" t="s">
-        <v>133</v>
+        <v>177</v>
       </c>
       <c r="H68" s="49" t="s">
         <v>377</v>
@@ -44825,30 +44963,14 @@
       <c r="AA68" s="4"/>
     </row>
     <row r="69" ht="22.5" customHeight="1">
-      <c r="A69" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="B69" s="47" t="s">
-        <v>372</v>
-      </c>
-      <c r="C69" s="48" t="s">
-        <v>309</v>
-      </c>
-      <c r="D69" s="48" t="s">
-        <v>310</v>
-      </c>
-      <c r="E69" s="49" t="s">
-        <v>376</v>
-      </c>
-      <c r="F69" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="G69" s="49" t="s">
-        <v>140</v>
-      </c>
-      <c r="H69" s="49" t="s">
-        <v>378</v>
-      </c>
+      <c r="A69" s="55"/>
+      <c r="B69" s="47"/>
+      <c r="C69" s="48"/>
+      <c r="D69" s="48"/>
+      <c r="E69" s="49"/>
+      <c r="F69" s="50"/>
+      <c r="G69" s="49"/>
+      <c r="H69" s="49"/>
       <c r="I69" s="4"/>
       <c r="J69" s="4"/>
       <c r="K69" s="4"/>
@@ -44870,14 +44992,30 @@
       <c r="AA69" s="4"/>
     </row>
     <row r="70" ht="22.5" customHeight="1">
-      <c r="A70" s="55"/>
-      <c r="B70" s="47"/>
-      <c r="C70" s="48"/>
-      <c r="D70" s="48"/>
-      <c r="E70" s="49"/>
-      <c r="F70" s="50"/>
-      <c r="G70" s="49"/>
-      <c r="H70" s="49"/>
+      <c r="A70" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B70" s="47" t="s">
+        <v>378</v>
+      </c>
+      <c r="C70" s="48" t="s">
+        <v>261</v>
+      </c>
+      <c r="D70" s="48" t="s">
+        <v>258</v>
+      </c>
+      <c r="E70" s="49" t="s">
+        <v>379</v>
+      </c>
+      <c r="F70" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="G70" s="49" t="s">
+        <v>124</v>
+      </c>
+      <c r="H70" s="49" t="s">
+        <v>380</v>
+      </c>
       <c r="I70" s="4"/>
       <c r="J70" s="4"/>
       <c r="K70" s="4"/>
@@ -44903,25 +45041,25 @@
         <v>16</v>
       </c>
       <c r="B71" s="47" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C71" s="48" t="s">
-        <v>261</v>
+        <v>306</v>
       </c>
       <c r="D71" s="48" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="E71" s="49" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F71" s="48" t="s">
         <v>26</v>
       </c>
       <c r="G71" s="49" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="H71" s="49" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="I71" s="4"/>
       <c r="J71" s="4"/>
@@ -44944,30 +45082,14 @@
       <c r="AA71" s="4"/>
     </row>
     <row r="72" ht="22.5" customHeight="1">
-      <c r="A72" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="B72" s="47" t="s">
-        <v>379</v>
-      </c>
-      <c r="C72" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="D72" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E72" s="49" t="s">
-        <v>382</v>
-      </c>
-      <c r="F72" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="G72" s="49" t="s">
-        <v>155</v>
-      </c>
-      <c r="H72" s="49" t="s">
-        <v>383</v>
-      </c>
+      <c r="A72" s="55"/>
+      <c r="B72" s="47"/>
+      <c r="C72" s="48"/>
+      <c r="D72" s="48"/>
+      <c r="E72" s="49"/>
+      <c r="F72" s="50"/>
+      <c r="G72" s="49"/>
+      <c r="H72" s="49"/>
       <c r="I72" s="4"/>
       <c r="J72" s="4"/>
       <c r="K72" s="4"/>
@@ -44993,13 +45115,13 @@
         <v>16</v>
       </c>
       <c r="B73" s="47" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="C73" s="48" t="s">
-        <v>306</v>
+        <v>257</v>
       </c>
       <c r="D73" s="48" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="E73" s="49" t="s">
         <v>384</v>
@@ -45008,9 +45130,9 @@
         <v>26</v>
       </c>
       <c r="G73" s="49" t="s">
-        <v>147</v>
-      </c>
-      <c r="H73" s="56" t="s">
+        <v>140</v>
+      </c>
+      <c r="H73" s="49" t="s">
         <v>385</v>
       </c>
       <c r="I73" s="4"/>
@@ -45038,7 +45160,7 @@
         <v>16</v>
       </c>
       <c r="B74" s="47" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="C74" s="48" t="s">
         <v>306</v>
@@ -45047,16 +45169,16 @@
         <v>262</v>
       </c>
       <c r="E74" s="49" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="F74" s="48" t="s">
         <v>26</v>
       </c>
       <c r="G74" s="49" t="s">
-        <v>147</v>
-      </c>
-      <c r="H74" s="56" t="s">
-        <v>387</v>
+        <v>124</v>
+      </c>
+      <c r="H74" s="49" t="s">
+        <v>386</v>
       </c>
       <c r="I74" s="4"/>
       <c r="J74" s="4"/>
@@ -45079,14 +45201,30 @@
       <c r="AA74" s="4"/>
     </row>
     <row r="75" ht="22.5" customHeight="1">
-      <c r="A75" s="50"/>
-      <c r="B75" s="49"/>
-      <c r="C75" s="48"/>
-      <c r="D75" s="48"/>
-      <c r="E75" s="58"/>
-      <c r="F75" s="50"/>
-      <c r="G75" s="49"/>
-      <c r="H75" s="49"/>
+      <c r="A75" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B75" s="47" t="s">
+        <v>383</v>
+      </c>
+      <c r="C75" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D75" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E75" s="49" t="s">
+        <v>387</v>
+      </c>
+      <c r="F75" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="G75" s="49" t="s">
+        <v>133</v>
+      </c>
+      <c r="H75" s="49" t="s">
+        <v>388</v>
+      </c>
       <c r="I75" s="4"/>
       <c r="J75" s="4"/>
       <c r="K75" s="4"/>
@@ -45108,29 +45246,29 @@
       <c r="AA75" s="4"/>
     </row>
     <row r="76" ht="22.5" customHeight="1">
-      <c r="A76" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B76" s="52" t="s">
-        <v>388</v>
+      <c r="A76" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B76" s="47" t="s">
+        <v>383</v>
       </c>
       <c r="C76" s="48" t="s">
-        <v>257</v>
+        <v>309</v>
       </c>
       <c r="D76" s="48" t="s">
-        <v>258</v>
+        <v>310</v>
       </c>
       <c r="E76" s="49" t="s">
+        <v>387</v>
+      </c>
+      <c r="F76" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="G76" s="49" t="s">
+        <v>140</v>
+      </c>
+      <c r="H76" s="49" t="s">
         <v>389</v>
-      </c>
-      <c r="F76" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="G76" s="49" t="s">
-        <v>100</v>
-      </c>
-      <c r="H76" s="49" t="s">
-        <v>390</v>
       </c>
       <c r="I76" s="4"/>
       <c r="J76" s="4"/>
@@ -45153,30 +45291,14 @@
       <c r="AA76" s="4"/>
     </row>
     <row r="77" ht="22.5" customHeight="1">
-      <c r="A77" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B77" s="52" t="s">
-        <v>388</v>
-      </c>
-      <c r="C77" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="D77" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E77" s="49" t="s">
-        <v>389</v>
-      </c>
-      <c r="F77" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="G77" s="49" t="s">
-        <v>100</v>
-      </c>
-      <c r="H77" s="49" t="s">
-        <v>391</v>
-      </c>
+      <c r="A77" s="55"/>
+      <c r="B77" s="47"/>
+      <c r="C77" s="48"/>
+      <c r="D77" s="48"/>
+      <c r="E77" s="49"/>
+      <c r="F77" s="50"/>
+      <c r="G77" s="49"/>
+      <c r="H77" s="49"/>
       <c r="I77" s="4"/>
       <c r="J77" s="4"/>
       <c r="K77" s="4"/>
@@ -45198,29 +45320,29 @@
       <c r="AA77" s="4"/>
     </row>
     <row r="78" ht="22.5" customHeight="1">
-      <c r="A78" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B78" s="52" t="s">
-        <v>388</v>
+      <c r="A78" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B78" s="47" t="s">
+        <v>390</v>
       </c>
       <c r="C78" s="48" t="s">
-        <v>306</v>
+        <v>261</v>
       </c>
       <c r="D78" s="48" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="E78" s="49" t="s">
+        <v>391</v>
+      </c>
+      <c r="F78" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="G78" s="49" t="s">
+        <v>147</v>
+      </c>
+      <c r="H78" s="49" t="s">
         <v>392</v>
-      </c>
-      <c r="F78" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="G78" s="49" t="s">
-        <v>100</v>
-      </c>
-      <c r="H78" s="49" t="s">
-        <v>393</v>
       </c>
       <c r="I78" s="4"/>
       <c r="J78" s="4"/>
@@ -45243,26 +45365,26 @@
       <c r="AA78" s="4"/>
     </row>
     <row r="79" ht="22.5" customHeight="1">
-      <c r="A79" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B79" s="52" t="s">
-        <v>388</v>
+      <c r="A79" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B79" s="47" t="s">
+        <v>390</v>
       </c>
       <c r="C79" s="48" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D79" s="48" t="s">
-        <v>310</v>
+        <v>262</v>
       </c>
       <c r="E79" s="49" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F79" s="48" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="G79" s="49" t="s">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="H79" s="49" t="s">
         <v>394</v>
@@ -45288,29 +45410,29 @@
       <c r="AA79" s="4"/>
     </row>
     <row r="80" ht="22.5" customHeight="1">
-      <c r="A80" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B80" s="52" t="s">
-        <v>388</v>
+      <c r="A80" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B80" s="47" t="s">
+        <v>390</v>
       </c>
       <c r="C80" s="48" t="s">
-        <v>336</v>
+        <v>306</v>
       </c>
       <c r="D80" s="48" t="s">
-        <v>337</v>
+        <v>262</v>
       </c>
       <c r="E80" s="49" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="F80" s="48" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="G80" s="49" t="s">
-        <v>100</v>
-      </c>
-      <c r="H80" s="49" t="s">
-        <v>395</v>
+        <v>147</v>
+      </c>
+      <c r="H80" s="58" t="s">
+        <v>396</v>
       </c>
       <c r="I80" s="4"/>
       <c r="J80" s="4"/>
@@ -45333,14 +45455,30 @@
       <c r="AA80" s="4"/>
     </row>
     <row r="81" ht="22.5" customHeight="1">
-      <c r="A81" s="59"/>
-      <c r="B81" s="52"/>
-      <c r="C81" s="48"/>
-      <c r="D81" s="48"/>
-      <c r="E81" s="49"/>
-      <c r="F81" s="50"/>
-      <c r="G81" s="49"/>
-      <c r="H81" s="49"/>
+      <c r="A81" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B81" s="47" t="s">
+        <v>390</v>
+      </c>
+      <c r="C81" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D81" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E81" s="49" t="s">
+        <v>397</v>
+      </c>
+      <c r="F81" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="G81" s="49" t="s">
+        <v>147</v>
+      </c>
+      <c r="H81" s="58" t="s">
+        <v>398</v>
+      </c>
       <c r="I81" s="4"/>
       <c r="J81" s="4"/>
       <c r="K81" s="4"/>
@@ -45362,30 +45500,14 @@
       <c r="AA81" s="4"/>
     </row>
     <row r="82" ht="22.5" customHeight="1">
-      <c r="A82" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B82" s="52" t="s">
-        <v>396</v>
-      </c>
-      <c r="C82" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="D82" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E82" s="49" t="s">
-        <v>397</v>
-      </c>
-      <c r="F82" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="G82" s="49" t="s">
-        <v>170</v>
-      </c>
-      <c r="H82" s="49" t="s">
-        <v>398</v>
-      </c>
+      <c r="A82" s="55"/>
+      <c r="B82" s="47"/>
+      <c r="C82" s="48"/>
+      <c r="D82" s="48"/>
+      <c r="E82" s="49"/>
+      <c r="F82" s="50"/>
+      <c r="G82" s="49"/>
+      <c r="H82" s="58"/>
       <c r="I82" s="4"/>
       <c r="J82" s="4"/>
       <c r="K82" s="4"/>
@@ -45407,29 +45529,29 @@
       <c r="AA82" s="4"/>
     </row>
     <row r="83" ht="22.5" customHeight="1">
-      <c r="A83" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B83" s="52" t="s">
-        <v>396</v>
-      </c>
-      <c r="C83" s="48" t="s">
-        <v>309</v>
-      </c>
-      <c r="D83" s="48" t="s">
-        <v>310</v>
-      </c>
-      <c r="E83" s="49" t="s">
-        <v>397</v>
-      </c>
-      <c r="F83" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="G83" s="49" t="s">
-        <v>170</v>
-      </c>
-      <c r="H83" s="49" t="s">
+      <c r="A83" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B83" s="47" t="s">
         <v>399</v>
+      </c>
+      <c r="C83" s="56" t="s">
+        <v>306</v>
+      </c>
+      <c r="D83" s="56" t="s">
+        <v>262</v>
+      </c>
+      <c r="E83" s="57" t="s">
+        <v>400</v>
+      </c>
+      <c r="F83" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="G83" s="57" t="s">
+        <v>116</v>
+      </c>
+      <c r="H83" s="57" t="s">
+        <v>401</v>
       </c>
       <c r="I83" s="4"/>
       <c r="J83" s="4"/>
@@ -45452,29 +45574,29 @@
       <c r="AA83" s="4"/>
     </row>
     <row r="84" ht="22.5" customHeight="1">
-      <c r="A84" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B84" s="52" t="s">
-        <v>396</v>
-      </c>
-      <c r="C84" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="D84" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E84" s="49" t="s">
-        <v>400</v>
-      </c>
-      <c r="F84" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="G84" s="49" t="s">
-        <v>163</v>
-      </c>
-      <c r="H84" s="49" t="s">
-        <v>401</v>
+      <c r="A84" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B84" s="47" t="s">
+        <v>399</v>
+      </c>
+      <c r="C84" s="56" t="s">
+        <v>261</v>
+      </c>
+      <c r="D84" s="56" t="s">
+        <v>258</v>
+      </c>
+      <c r="E84" s="57" t="s">
+        <v>402</v>
+      </c>
+      <c r="F84" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="G84" s="57" t="s">
+        <v>116</v>
+      </c>
+      <c r="H84" s="57" t="s">
+        <v>403</v>
       </c>
       <c r="I84" s="4"/>
       <c r="J84" s="4"/>
@@ -45497,14 +45619,30 @@
       <c r="AA84" s="4"/>
     </row>
     <row r="85" ht="22.5" customHeight="1">
-      <c r="A85" s="59"/>
-      <c r="B85" s="52"/>
-      <c r="C85" s="48"/>
-      <c r="D85" s="48"/>
-      <c r="E85" s="49"/>
-      <c r="F85" s="50"/>
-      <c r="G85" s="49"/>
-      <c r="H85" s="49"/>
+      <c r="A85" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B85" s="47" t="s">
+        <v>399</v>
+      </c>
+      <c r="C85" s="56" t="s">
+        <v>261</v>
+      </c>
+      <c r="D85" s="56" t="s">
+        <v>258</v>
+      </c>
+      <c r="E85" s="57" t="s">
+        <v>404</v>
+      </c>
+      <c r="F85" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="G85" s="57" t="s">
+        <v>116</v>
+      </c>
+      <c r="H85" s="57" t="s">
+        <v>405</v>
+      </c>
       <c r="I85" s="4"/>
       <c r="J85" s="4"/>
       <c r="K85" s="4"/>
@@ -45526,29 +45664,29 @@
       <c r="AA85" s="4"/>
     </row>
     <row r="86" ht="22.5" customHeight="1">
-      <c r="A86" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B86" s="52" t="s">
-        <v>402</v>
-      </c>
-      <c r="C86" s="48" t="s">
+      <c r="A86" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B86" s="47" t="s">
+        <v>399</v>
+      </c>
+      <c r="C86" s="56" t="s">
         <v>306</v>
       </c>
-      <c r="D86" s="48" t="s">
+      <c r="D86" s="56" t="s">
         <v>262</v>
       </c>
-      <c r="E86" s="49" t="s">
-        <v>403</v>
-      </c>
-      <c r="F86" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="G86" s="49" t="s">
-        <v>170</v>
-      </c>
-      <c r="H86" s="49" t="s">
-        <v>404</v>
+      <c r="E86" s="57" t="s">
+        <v>406</v>
+      </c>
+      <c r="F86" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="G86" s="57" t="s">
+        <v>116</v>
+      </c>
+      <c r="H86" s="57" t="s">
+        <v>407</v>
       </c>
       <c r="I86" s="4"/>
       <c r="J86" s="4"/>
@@ -45571,29 +45709,29 @@
       <c r="AA86" s="4"/>
     </row>
     <row r="87" ht="22.5" customHeight="1">
-      <c r="A87" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B87" s="52" t="s">
-        <v>402</v>
-      </c>
-      <c r="C87" s="48" t="s">
-        <v>261</v>
-      </c>
-      <c r="D87" s="48" t="s">
-        <v>258</v>
-      </c>
-      <c r="E87" s="49" t="s">
-        <v>405</v>
-      </c>
-      <c r="F87" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="G87" s="49" t="s">
-        <v>170</v>
-      </c>
-      <c r="H87" s="49" t="s">
-        <v>406</v>
+      <c r="A87" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="B87" s="47" t="s">
+        <v>399</v>
+      </c>
+      <c r="C87" s="56" t="s">
+        <v>336</v>
+      </c>
+      <c r="D87" s="56" t="s">
+        <v>337</v>
+      </c>
+      <c r="E87" s="57" t="s">
+        <v>408</v>
+      </c>
+      <c r="F87" s="56" t="s">
+        <v>26</v>
+      </c>
+      <c r="G87" s="57" t="s">
+        <v>116</v>
+      </c>
+      <c r="H87" s="57" t="s">
+        <v>409</v>
       </c>
       <c r="I87" s="4"/>
       <c r="J87" s="4"/>
@@ -45620,7 +45758,7 @@
       <c r="B88" s="49"/>
       <c r="C88" s="48"/>
       <c r="D88" s="48"/>
-      <c r="E88" s="49"/>
+      <c r="E88" s="59"/>
       <c r="F88" s="50"/>
       <c r="G88" s="49"/>
       <c r="H88" s="49"/>
@@ -45645,29 +45783,29 @@
       <c r="AA88" s="4"/>
     </row>
     <row r="89" ht="22.5" customHeight="1">
-      <c r="A89" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B89" s="54" t="s">
-        <v>407</v>
+      <c r="A89" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="B89" s="52" t="s">
+        <v>410</v>
       </c>
       <c r="C89" s="48" t="s">
-        <v>306</v>
+        <v>257</v>
       </c>
       <c r="D89" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E89" s="57" t="s">
-        <v>408</v>
+        <v>258</v>
+      </c>
+      <c r="E89" s="49" t="s">
+        <v>411</v>
       </c>
       <c r="F89" s="48" t="s">
-        <v>76</v>
+        <v>37</v>
       </c>
       <c r="G89" s="49" t="s">
-        <v>198</v>
-      </c>
-      <c r="H89" s="57" t="s">
-        <v>409</v>
+        <v>100</v>
+      </c>
+      <c r="H89" s="49" t="s">
+        <v>412</v>
       </c>
       <c r="I89" s="4"/>
       <c r="J89" s="4"/>
@@ -45690,14 +45828,30 @@
       <c r="AA89" s="4"/>
     </row>
     <row r="90" ht="22.5" customHeight="1">
-      <c r="A90" s="60"/>
-      <c r="B90" s="54"/>
-      <c r="C90" s="48"/>
-      <c r="D90" s="48"/>
-      <c r="E90" s="57"/>
-      <c r="F90" s="50"/>
-      <c r="G90" s="49"/>
-      <c r="H90" s="57"/>
+      <c r="A90" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="B90" s="52" t="s">
+        <v>410</v>
+      </c>
+      <c r="C90" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D90" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E90" s="49" t="s">
+        <v>411</v>
+      </c>
+      <c r="F90" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="G90" s="49" t="s">
+        <v>100</v>
+      </c>
+      <c r="H90" s="49" t="s">
+        <v>413</v>
+      </c>
       <c r="I90" s="4"/>
       <c r="J90" s="4"/>
       <c r="K90" s="4"/>
@@ -45719,10 +45873,10 @@
       <c r="AA90" s="4"/>
     </row>
     <row r="91" ht="22.5" customHeight="1">
-      <c r="A91" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B91" s="54" t="s">
+      <c r="A91" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="B91" s="52" t="s">
         <v>410</v>
       </c>
       <c r="C91" s="48" t="s">
@@ -45731,17 +45885,17 @@
       <c r="D91" s="48" t="s">
         <v>262</v>
       </c>
-      <c r="E91" s="57" t="s">
-        <v>411</v>
+      <c r="E91" s="49" t="s">
+        <v>414</v>
       </c>
       <c r="F91" s="48" t="s">
-        <v>162</v>
+        <v>37</v>
       </c>
       <c r="G91" s="49" t="s">
-        <v>213</v>
-      </c>
-      <c r="H91" s="57" t="s">
-        <v>412</v>
+        <v>100</v>
+      </c>
+      <c r="H91" s="49" t="s">
+        <v>415</v>
       </c>
       <c r="I91" s="4"/>
       <c r="J91" s="4"/>
@@ -45764,10 +45918,10 @@
       <c r="AA91" s="4"/>
     </row>
     <row r="92" ht="22.5" customHeight="1">
-      <c r="A92" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B92" s="54" t="s">
+      <c r="A92" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="B92" s="52" t="s">
         <v>410</v>
       </c>
       <c r="C92" s="48" t="s">
@@ -45776,17 +45930,17 @@
       <c r="D92" s="48" t="s">
         <v>310</v>
       </c>
-      <c r="E92" s="57" t="s">
-        <v>413</v>
+      <c r="E92" s="49" t="s">
+        <v>414</v>
       </c>
       <c r="F92" s="48" t="s">
-        <v>162</v>
+        <v>37</v>
       </c>
       <c r="G92" s="49" t="s">
-        <v>213</v>
-      </c>
-      <c r="H92" s="57" t="s">
-        <v>414</v>
+        <v>100</v>
+      </c>
+      <c r="H92" s="49" t="s">
+        <v>416</v>
       </c>
       <c r="I92" s="4"/>
       <c r="J92" s="4"/>
@@ -45809,29 +45963,29 @@
       <c r="AA92" s="4"/>
     </row>
     <row r="93" ht="22.5" customHeight="1">
-      <c r="A93" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B93" s="54" t="s">
+      <c r="A93" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="B93" s="52" t="s">
         <v>410</v>
       </c>
       <c r="C93" s="48" t="s">
-        <v>306</v>
+        <v>336</v>
       </c>
       <c r="D93" s="48" t="s">
-        <v>262</v>
+        <v>337</v>
       </c>
       <c r="E93" s="49" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F93" s="48" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="G93" s="49" t="s">
-        <v>206</v>
+        <v>100</v>
       </c>
       <c r="H93" s="49" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="I93" s="4"/>
       <c r="J93" s="4"/>
@@ -45854,30 +46008,14 @@
       <c r="AA93" s="4"/>
     </row>
     <row r="94" ht="22.5" customHeight="1">
-      <c r="A94" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B94" s="54" t="s">
-        <v>410</v>
-      </c>
-      <c r="C94" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="D94" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E94" s="49" t="s">
-        <v>417</v>
-      </c>
-      <c r="F94" s="48" t="s">
-        <v>162</v>
-      </c>
-      <c r="G94" s="49" t="s">
-        <v>213</v>
-      </c>
-      <c r="H94" s="49" t="s">
-        <v>418</v>
-      </c>
+      <c r="A94" s="60"/>
+      <c r="B94" s="52"/>
+      <c r="C94" s="48"/>
+      <c r="D94" s="48"/>
+      <c r="E94" s="49"/>
+      <c r="F94" s="50"/>
+      <c r="G94" s="49"/>
+      <c r="H94" s="49"/>
       <c r="I94" s="4"/>
       <c r="J94" s="4"/>
       <c r="K94" s="4"/>
@@ -45899,26 +46037,26 @@
       <c r="AA94" s="4"/>
     </row>
     <row r="95" ht="22.5" customHeight="1">
-      <c r="A95" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B95" s="54" t="s">
-        <v>410</v>
+      <c r="A95" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="B95" s="52" t="s">
+        <v>418</v>
       </c>
       <c r="C95" s="48" t="s">
-        <v>261</v>
+        <v>306</v>
       </c>
       <c r="D95" s="48" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="E95" s="49" t="s">
         <v>419</v>
       </c>
       <c r="F95" s="48" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="G95" s="49" t="s">
-        <v>206</v>
+        <v>170</v>
       </c>
       <c r="H95" s="49" t="s">
         <v>420</v>
@@ -45944,29 +46082,29 @@
       <c r="AA95" s="4"/>
     </row>
     <row r="96" ht="22.5" customHeight="1">
-      <c r="A96" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B96" s="54" t="s">
-        <v>410</v>
+      <c r="A96" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="B96" s="52" t="s">
+        <v>418</v>
       </c>
       <c r="C96" s="48" t="s">
-        <v>261</v>
+        <v>309</v>
       </c>
       <c r="D96" s="48" t="s">
-        <v>258</v>
+        <v>310</v>
       </c>
       <c r="E96" s="49" t="s">
+        <v>419</v>
+      </c>
+      <c r="F96" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="G96" s="49" t="s">
+        <v>170</v>
+      </c>
+      <c r="H96" s="49" t="s">
         <v>421</v>
-      </c>
-      <c r="F96" s="48" t="s">
-        <v>25</v>
-      </c>
-      <c r="G96" s="49" t="s">
-        <v>206</v>
-      </c>
-      <c r="H96" s="49" t="s">
-        <v>422</v>
       </c>
       <c r="I96" s="4"/>
       <c r="J96" s="4"/>
@@ -45989,14 +46127,30 @@
       <c r="AA96" s="4"/>
     </row>
     <row r="97" ht="22.5" customHeight="1">
-      <c r="A97" s="60"/>
-      <c r="B97" s="54"/>
-      <c r="C97" s="48"/>
-      <c r="D97" s="48"/>
-      <c r="E97" s="49"/>
-      <c r="F97" s="50"/>
-      <c r="G97" s="49"/>
-      <c r="H97" s="49"/>
+      <c r="A97" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="B97" s="52" t="s">
+        <v>418</v>
+      </c>
+      <c r="C97" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D97" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E97" s="49" t="s">
+        <v>422</v>
+      </c>
+      <c r="F97" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="G97" s="49" t="s">
+        <v>163</v>
+      </c>
+      <c r="H97" s="49" t="s">
+        <v>423</v>
+      </c>
       <c r="I97" s="4"/>
       <c r="J97" s="4"/>
       <c r="K97" s="4"/>
@@ -46018,30 +46172,14 @@
       <c r="AA97" s="4"/>
     </row>
     <row r="98" ht="22.5" customHeight="1">
-      <c r="A98" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B98" s="54" t="s">
-        <v>423</v>
-      </c>
-      <c r="C98" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="D98" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E98" s="49" t="s">
-        <v>424</v>
-      </c>
-      <c r="F98" s="48" t="s">
-        <v>25</v>
-      </c>
-      <c r="G98" s="49" t="s">
-        <v>232</v>
-      </c>
-      <c r="H98" s="49" t="s">
-        <v>425</v>
-      </c>
+      <c r="A98" s="60"/>
+      <c r="B98" s="52"/>
+      <c r="C98" s="48"/>
+      <c r="D98" s="48"/>
+      <c r="E98" s="49"/>
+      <c r="F98" s="50"/>
+      <c r="G98" s="49"/>
+      <c r="H98" s="49"/>
       <c r="I98" s="4"/>
       <c r="J98" s="4"/>
       <c r="K98" s="4"/>
@@ -46063,11 +46201,11 @@
       <c r="AA98" s="4"/>
     </row>
     <row r="99" ht="22.5" customHeight="1">
-      <c r="A99" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B99" s="54" t="s">
-        <v>423</v>
+      <c r="A99" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="B99" s="52" t="s">
+        <v>424</v>
       </c>
       <c r="C99" s="48" t="s">
         <v>306</v>
@@ -46076,16 +46214,16 @@
         <v>262</v>
       </c>
       <c r="E99" s="49" t="s">
+        <v>425</v>
+      </c>
+      <c r="F99" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="G99" s="49" t="s">
+        <v>170</v>
+      </c>
+      <c r="H99" s="49" t="s">
         <v>426</v>
-      </c>
-      <c r="F99" s="48" t="s">
-        <v>25</v>
-      </c>
-      <c r="G99" s="49" t="s">
-        <v>232</v>
-      </c>
-      <c r="H99" s="49" t="s">
-        <v>427</v>
       </c>
       <c r="I99" s="4"/>
       <c r="J99" s="4"/>
@@ -46108,29 +46246,29 @@
       <c r="AA99" s="4"/>
     </row>
     <row r="100" ht="22.5" customHeight="1">
-      <c r="A100" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B100" s="54" t="s">
-        <v>423</v>
+      <c r="A100" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="B100" s="52" t="s">
+        <v>424</v>
       </c>
       <c r="C100" s="48" t="s">
-        <v>309</v>
+        <v>261</v>
       </c>
       <c r="D100" s="48" t="s">
-        <v>310</v>
+        <v>258</v>
       </c>
       <c r="E100" s="49" t="s">
+        <v>427</v>
+      </c>
+      <c r="F100" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="G100" s="49" t="s">
+        <v>170</v>
+      </c>
+      <c r="H100" s="49" t="s">
         <v>428</v>
-      </c>
-      <c r="F100" s="48" t="s">
-        <v>25</v>
-      </c>
-      <c r="G100" s="49" t="s">
-        <v>232</v>
-      </c>
-      <c r="H100" s="49" t="s">
-        <v>429</v>
       </c>
       <c r="I100" s="4"/>
       <c r="J100" s="4"/>
@@ -46153,8 +46291,8 @@
       <c r="AA100" s="4"/>
     </row>
     <row r="101" ht="22.5" customHeight="1">
-      <c r="A101" s="60"/>
-      <c r="B101" s="54"/>
+      <c r="A101" s="50"/>
+      <c r="B101" s="49"/>
       <c r="C101" s="48"/>
       <c r="D101" s="48"/>
       <c r="E101" s="49"/>
@@ -46186,7 +46324,7 @@
         <v>200</v>
       </c>
       <c r="B102" s="54" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C102" s="48" t="s">
         <v>306</v>
@@ -46194,17 +46332,17 @@
       <c r="D102" s="48" t="s">
         <v>262</v>
       </c>
-      <c r="E102" s="57" t="s">
+      <c r="E102" s="49" t="s">
+        <v>430</v>
+      </c>
+      <c r="F102" s="48" t="s">
+        <v>76</v>
+      </c>
+      <c r="G102" s="49" t="s">
+        <v>198</v>
+      </c>
+      <c r="H102" s="49" t="s">
         <v>431</v>
-      </c>
-      <c r="F102" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="G102" s="49" t="s">
-        <v>220</v>
-      </c>
-      <c r="H102" s="49" t="s">
-        <v>432</v>
       </c>
       <c r="I102" s="4"/>
       <c r="J102" s="4"/>
@@ -46227,30 +46365,14 @@
       <c r="AA102" s="4"/>
     </row>
     <row r="103" ht="22.5" customHeight="1">
-      <c r="A103" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B103" s="54" t="s">
-        <v>430</v>
-      </c>
-      <c r="C103" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="D103" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E103" s="49" t="s">
-        <v>433</v>
-      </c>
-      <c r="F103" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="G103" s="49" t="s">
-        <v>220</v>
-      </c>
-      <c r="H103" s="49" t="s">
-        <v>434</v>
-      </c>
+      <c r="A103" s="61"/>
+      <c r="B103" s="54"/>
+      <c r="C103" s="48"/>
+      <c r="D103" s="48"/>
+      <c r="E103" s="49"/>
+      <c r="F103" s="50"/>
+      <c r="G103" s="49"/>
+      <c r="H103" s="49"/>
       <c r="I103" s="4"/>
       <c r="J103" s="4"/>
       <c r="K103" s="4"/>
@@ -46276,25 +46398,25 @@
         <v>200</v>
       </c>
       <c r="B104" s="54" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="C104" s="48" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D104" s="48" t="s">
-        <v>310</v>
-      </c>
-      <c r="E104" s="57" t="s">
-        <v>435</v>
+        <v>262</v>
+      </c>
+      <c r="E104" s="49" t="s">
+        <v>433</v>
       </c>
       <c r="F104" s="48" t="s">
-        <v>37</v>
+        <v>162</v>
       </c>
       <c r="G104" s="49" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="H104" s="49" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="I104" s="4"/>
       <c r="J104" s="4"/>
@@ -46317,14 +46439,30 @@
       <c r="AA104" s="4"/>
     </row>
     <row r="105" ht="22.5" customHeight="1">
-      <c r="A105" s="60"/>
-      <c r="B105" s="54"/>
-      <c r="C105" s="48"/>
-      <c r="D105" s="48"/>
-      <c r="E105" s="49"/>
-      <c r="F105" s="50"/>
-      <c r="G105" s="49"/>
-      <c r="H105" s="49"/>
+      <c r="A105" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B105" s="54" t="s">
+        <v>432</v>
+      </c>
+      <c r="C105" s="48" t="s">
+        <v>309</v>
+      </c>
+      <c r="D105" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="E105" s="49" t="s">
+        <v>435</v>
+      </c>
+      <c r="F105" s="48" t="s">
+        <v>162</v>
+      </c>
+      <c r="G105" s="49" t="s">
+        <v>213</v>
+      </c>
+      <c r="H105" s="49" t="s">
+        <v>436</v>
+      </c>
       <c r="I105" s="4"/>
       <c r="J105" s="4"/>
       <c r="K105" s="4"/>
@@ -46350,7 +46488,7 @@
         <v>200</v>
       </c>
       <c r="B106" s="54" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="C106" s="48" t="s">
         <v>306</v>
@@ -46358,17 +46496,17 @@
       <c r="D106" s="48" t="s">
         <v>262</v>
       </c>
-      <c r="E106" s="57" t="s">
+      <c r="E106" s="49" t="s">
+        <v>437</v>
+      </c>
+      <c r="F106" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="G106" s="49" t="s">
+        <v>206</v>
+      </c>
+      <c r="H106" s="49" t="s">
         <v>438</v>
-      </c>
-      <c r="F106" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="G106" s="49" t="s">
-        <v>226</v>
-      </c>
-      <c r="H106" s="49" t="s">
-        <v>439</v>
       </c>
       <c r="I106" s="4"/>
       <c r="J106" s="4"/>
@@ -46395,7 +46533,7 @@
         <v>200</v>
       </c>
       <c r="B107" s="54" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="C107" s="48" t="s">
         <v>306</v>
@@ -46404,16 +46542,16 @@
         <v>262</v>
       </c>
       <c r="E107" s="49" t="s">
+        <v>439</v>
+      </c>
+      <c r="F107" s="48" t="s">
+        <v>162</v>
+      </c>
+      <c r="G107" s="49" t="s">
+        <v>213</v>
+      </c>
+      <c r="H107" s="49" t="s">
         <v>440</v>
-      </c>
-      <c r="F107" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="G107" s="49" t="s">
-        <v>226</v>
-      </c>
-      <c r="H107" s="49" t="s">
-        <v>441</v>
       </c>
       <c r="I107" s="4"/>
       <c r="J107" s="4"/>
@@ -46436,14 +46574,30 @@
       <c r="AA107" s="4"/>
     </row>
     <row r="108" ht="22.5" customHeight="1">
-      <c r="A108" s="60"/>
-      <c r="B108" s="54"/>
-      <c r="C108" s="48"/>
-      <c r="D108" s="48"/>
-      <c r="E108" s="49"/>
-      <c r="F108" s="50"/>
-      <c r="G108" s="49"/>
-      <c r="H108" s="49"/>
+      <c r="A108" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B108" s="54" t="s">
+        <v>432</v>
+      </c>
+      <c r="C108" s="48" t="s">
+        <v>261</v>
+      </c>
+      <c r="D108" s="48" t="s">
+        <v>258</v>
+      </c>
+      <c r="E108" s="49" t="s">
+        <v>441</v>
+      </c>
+      <c r="F108" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="G108" s="49" t="s">
+        <v>206</v>
+      </c>
+      <c r="H108" s="49" t="s">
+        <v>442</v>
+      </c>
       <c r="I108" s="4"/>
       <c r="J108" s="4"/>
       <c r="K108" s="4"/>
@@ -46469,24 +46623,24 @@
         <v>200</v>
       </c>
       <c r="B109" s="54" t="s">
-        <v>442</v>
+        <v>432</v>
       </c>
       <c r="C109" s="48" t="s">
-        <v>306</v>
+        <v>261</v>
       </c>
       <c r="D109" s="48" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="E109" s="49" t="s">
         <v>443</v>
       </c>
       <c r="F109" s="48" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="G109" s="49" t="s">
-        <v>226</v>
-      </c>
-      <c r="H109" s="57" t="s">
+        <v>206</v>
+      </c>
+      <c r="H109" s="49" t="s">
         <v>444</v>
       </c>
       <c r="I109" s="4"/>
@@ -46510,30 +46664,14 @@
       <c r="AA109" s="4"/>
     </row>
     <row r="110" ht="22.5" customHeight="1">
-      <c r="A110" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B110" s="54" t="s">
-        <v>442</v>
-      </c>
-      <c r="C110" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="D110" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E110" s="49" t="s">
-        <v>445</v>
-      </c>
-      <c r="F110" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="G110" s="49" t="s">
-        <v>226</v>
-      </c>
-      <c r="H110" s="57" t="s">
-        <v>446</v>
-      </c>
+      <c r="A110" s="61"/>
+      <c r="B110" s="54"/>
+      <c r="C110" s="48"/>
+      <c r="D110" s="48"/>
+      <c r="E110" s="49"/>
+      <c r="F110" s="50"/>
+      <c r="G110" s="49"/>
+      <c r="H110" s="49"/>
       <c r="I110" s="4"/>
       <c r="J110" s="4"/>
       <c r="K110" s="4"/>
@@ -46559,25 +46697,25 @@
         <v>200</v>
       </c>
       <c r="B111" s="54" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="C111" s="48" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D111" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E111" s="49" t="s">
+        <v>446</v>
+      </c>
+      <c r="F111" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="G111" s="49" t="s">
+        <v>232</v>
+      </c>
+      <c r="H111" s="49" t="s">
         <v>447</v>
-      </c>
-      <c r="E111" s="49" t="s">
-        <v>445</v>
-      </c>
-      <c r="F111" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="G111" s="49" t="s">
-        <v>226</v>
-      </c>
-      <c r="H111" s="57" t="s">
-        <v>448</v>
       </c>
       <c r="I111" s="4"/>
       <c r="J111" s="4"/>
@@ -46604,7 +46742,7 @@
         <v>200</v>
       </c>
       <c r="B112" s="54" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="C112" s="48" t="s">
         <v>306</v>
@@ -46613,16 +46751,16 @@
         <v>262</v>
       </c>
       <c r="E112" s="49" t="s">
+        <v>448</v>
+      </c>
+      <c r="F112" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="G112" s="49" t="s">
+        <v>232</v>
+      </c>
+      <c r="H112" s="49" t="s">
         <v>449</v>
-      </c>
-      <c r="F112" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="G112" s="49" t="s">
-        <v>226</v>
-      </c>
-      <c r="H112" s="49" t="s">
-        <v>450</v>
       </c>
       <c r="I112" s="4"/>
       <c r="J112" s="4"/>
@@ -46645,14 +46783,30 @@
       <c r="AA112" s="4"/>
     </row>
     <row r="113" ht="22.5" customHeight="1">
-      <c r="A113" s="60"/>
-      <c r="B113" s="54"/>
-      <c r="C113" s="48"/>
-      <c r="D113" s="48"/>
-      <c r="E113" s="49"/>
-      <c r="F113" s="50"/>
-      <c r="G113" s="49"/>
-      <c r="H113" s="49"/>
+      <c r="A113" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B113" s="54" t="s">
+        <v>445</v>
+      </c>
+      <c r="C113" s="48" t="s">
+        <v>309</v>
+      </c>
+      <c r="D113" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="E113" s="49" t="s">
+        <v>450</v>
+      </c>
+      <c r="F113" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="G113" s="49" t="s">
+        <v>232</v>
+      </c>
+      <c r="H113" s="49" t="s">
+        <v>451</v>
+      </c>
       <c r="I113" s="4"/>
       <c r="J113" s="4"/>
       <c r="K113" s="4"/>
@@ -46674,30 +46828,14 @@
       <c r="AA113" s="4"/>
     </row>
     <row r="114" ht="22.5" customHeight="1">
-      <c r="A114" s="53" t="s">
-        <v>200</v>
-      </c>
-      <c r="B114" s="54" t="s">
-        <v>451</v>
-      </c>
-      <c r="C114" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="D114" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E114" s="49" t="s">
-        <v>452</v>
-      </c>
-      <c r="F114" s="48" t="s">
-        <v>47</v>
-      </c>
-      <c r="G114" s="49" t="s">
-        <v>239</v>
-      </c>
-      <c r="H114" s="49" t="s">
-        <v>453</v>
-      </c>
+      <c r="A114" s="61"/>
+      <c r="B114" s="54"/>
+      <c r="C114" s="48"/>
+      <c r="D114" s="48"/>
+      <c r="E114" s="49"/>
+      <c r="F114" s="50"/>
+      <c r="G114" s="49"/>
+      <c r="H114" s="49"/>
       <c r="I114" s="4"/>
       <c r="J114" s="4"/>
       <c r="K114" s="4"/>
@@ -46723,7 +46861,7 @@
         <v>200</v>
       </c>
       <c r="B115" s="54" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C115" s="48" t="s">
         <v>306</v>
@@ -46732,16 +46870,16 @@
         <v>262</v>
       </c>
       <c r="E115" s="49" t="s">
+        <v>453</v>
+      </c>
+      <c r="F115" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="G115" s="49" t="s">
+        <v>220</v>
+      </c>
+      <c r="H115" s="49" t="s">
         <v>454</v>
-      </c>
-      <c r="F115" s="48" t="s">
-        <v>47</v>
-      </c>
-      <c r="G115" s="49" t="s">
-        <v>239</v>
-      </c>
-      <c r="H115" s="49" t="s">
-        <v>455</v>
       </c>
       <c r="I115" s="4"/>
       <c r="J115" s="4"/>
@@ -46768,22 +46906,22 @@
         <v>200</v>
       </c>
       <c r="B116" s="54" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C116" s="48" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D116" s="48" t="s">
-        <v>310</v>
+        <v>262</v>
       </c>
       <c r="E116" s="49" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="F116" s="48" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="G116" s="49" t="s">
-        <v>239</v>
+        <v>220</v>
       </c>
       <c r="H116" s="49" t="s">
         <v>456</v>
@@ -46809,14 +46947,30 @@
       <c r="AA116" s="4"/>
     </row>
     <row r="117" ht="22.5" customHeight="1">
-      <c r="A117" s="50"/>
-      <c r="B117" s="49"/>
-      <c r="C117" s="48"/>
-      <c r="D117" s="48"/>
-      <c r="E117" s="49"/>
-      <c r="F117" s="50"/>
-      <c r="G117" s="49"/>
-      <c r="H117" s="49"/>
+      <c r="A117" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B117" s="54" t="s">
+        <v>452</v>
+      </c>
+      <c r="C117" s="48" t="s">
+        <v>309</v>
+      </c>
+      <c r="D117" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="E117" s="49" t="s">
+        <v>457</v>
+      </c>
+      <c r="F117" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="G117" s="49" t="s">
+        <v>220</v>
+      </c>
+      <c r="H117" s="49" t="s">
+        <v>458</v>
+      </c>
       <c r="I117" s="4"/>
       <c r="J117" s="4"/>
       <c r="K117" s="4"/>
@@ -46838,30 +46992,14 @@
       <c r="AA117" s="4"/>
     </row>
     <row r="118" ht="22.5" customHeight="1">
-      <c r="A118" s="48" t="s">
-        <v>457</v>
-      </c>
-      <c r="B118" s="49" t="s">
-        <v>458</v>
-      </c>
-      <c r="C118" s="48" t="s">
-        <v>306</v>
-      </c>
-      <c r="D118" s="48" t="s">
-        <v>262</v>
-      </c>
-      <c r="E118" s="49" t="s">
-        <v>459</v>
-      </c>
-      <c r="F118" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="G118" s="49" t="s">
-        <v>109</v>
-      </c>
-      <c r="H118" s="49" t="s">
-        <v>460</v>
-      </c>
+      <c r="A118" s="61"/>
+      <c r="B118" s="54"/>
+      <c r="C118" s="48"/>
+      <c r="D118" s="48"/>
+      <c r="E118" s="49"/>
+      <c r="F118" s="50"/>
+      <c r="G118" s="49"/>
+      <c r="H118" s="49"/>
       <c r="I118" s="4"/>
       <c r="J118" s="4"/>
       <c r="K118" s="4"/>
@@ -46883,11 +47021,11 @@
       <c r="AA118" s="4"/>
     </row>
     <row r="119" ht="22.5" customHeight="1">
-      <c r="A119" s="48" t="s">
-        <v>457</v>
-      </c>
-      <c r="B119" s="49" t="s">
-        <v>458</v>
+      <c r="A119" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B119" s="54" t="s">
+        <v>459</v>
       </c>
       <c r="C119" s="48" t="s">
         <v>306</v>
@@ -46896,16 +47034,16 @@
         <v>262</v>
       </c>
       <c r="E119" s="49" t="s">
+        <v>460</v>
+      </c>
+      <c r="F119" s="48" t="s">
+        <v>36</v>
+      </c>
+      <c r="G119" s="49" t="s">
+        <v>226</v>
+      </c>
+      <c r="H119" s="49" t="s">
         <v>461</v>
-      </c>
-      <c r="F119" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="G119" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="H119" s="49" t="s">
-        <v>462</v>
       </c>
       <c r="I119" s="4"/>
       <c r="J119" s="4"/>
@@ -46928,11 +47066,11 @@
       <c r="AA119" s="4"/>
     </row>
     <row r="120" ht="22.5" customHeight="1">
-      <c r="A120" s="48" t="s">
-        <v>457</v>
-      </c>
-      <c r="B120" s="49" t="s">
-        <v>463</v>
+      <c r="A120" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B120" s="54" t="s">
+        <v>459</v>
       </c>
       <c r="C120" s="48" t="s">
         <v>306</v>
@@ -46941,16 +47079,16 @@
         <v>262</v>
       </c>
       <c r="E120" s="49" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="F120" s="48" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G120" s="49" t="s">
-        <v>100</v>
+        <v>226</v>
       </c>
       <c r="H120" s="49" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="I120" s="4"/>
       <c r="J120" s="4"/>
@@ -46973,8 +47111,8 @@
       <c r="AA120" s="4"/>
     </row>
     <row r="121" ht="22.5" customHeight="1">
-      <c r="A121" s="50"/>
-      <c r="B121" s="49"/>
+      <c r="A121" s="61"/>
+      <c r="B121" s="54"/>
       <c r="C121" s="48"/>
       <c r="D121" s="48"/>
       <c r="E121" s="49"/>
@@ -47002,11 +47140,11 @@
       <c r="AA121" s="4"/>
     </row>
     <row r="122" ht="22.5" customHeight="1">
-      <c r="A122" s="48" t="s">
-        <v>466</v>
-      </c>
-      <c r="B122" s="49" t="s">
-        <v>467</v>
+      <c r="A122" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B122" s="54" t="s">
+        <v>464</v>
       </c>
       <c r="C122" s="48" t="s">
         <v>306</v>
@@ -47015,7 +47153,7 @@
         <v>262</v>
       </c>
       <c r="E122" s="49" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="F122" s="48" t="s">
         <v>36</v>
@@ -47024,7 +47162,7 @@
         <v>226</v>
       </c>
       <c r="H122" s="49" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="I122" s="4"/>
       <c r="J122" s="4"/>
@@ -47047,11 +47185,11 @@
       <c r="AA122" s="4"/>
     </row>
     <row r="123" ht="22.5" customHeight="1">
-      <c r="A123" s="48" t="s">
-        <v>466</v>
-      </c>
-      <c r="B123" s="49" t="s">
-        <v>467</v>
+      <c r="A123" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B123" s="54" t="s">
+        <v>464</v>
       </c>
       <c r="C123" s="48" t="s">
         <v>306</v>
@@ -47060,7 +47198,7 @@
         <v>262</v>
       </c>
       <c r="E123" s="49" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="F123" s="48" t="s">
         <v>36</v>
@@ -47069,7 +47207,7 @@
         <v>226</v>
       </c>
       <c r="H123" s="49" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="I123" s="4"/>
       <c r="J123" s="4"/>
@@ -47091,15 +47229,31 @@
       <c r="Z123" s="4"/>
       <c r="AA123" s="4"/>
     </row>
-    <row r="124">
-      <c r="A124" s="4"/>
-      <c r="B124" s="4"/>
-      <c r="C124" s="4"/>
-      <c r="D124" s="4"/>
-      <c r="E124" s="4"/>
-      <c r="F124" s="4"/>
-      <c r="G124" s="4"/>
-      <c r="H124" s="4"/>
+    <row r="124" ht="22.5" customHeight="1">
+      <c r="A124" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B124" s="54" t="s">
+        <v>464</v>
+      </c>
+      <c r="C124" s="48" t="s">
+        <v>309</v>
+      </c>
+      <c r="D124" s="48" t="s">
+        <v>469</v>
+      </c>
+      <c r="E124" s="49" t="s">
+        <v>467</v>
+      </c>
+      <c r="F124" s="48" t="s">
+        <v>36</v>
+      </c>
+      <c r="G124" s="49" t="s">
+        <v>226</v>
+      </c>
+      <c r="H124" s="49" t="s">
+        <v>470</v>
+      </c>
       <c r="I124" s="4"/>
       <c r="J124" s="4"/>
       <c r="K124" s="4"/>
@@ -47120,15 +47274,31 @@
       <c r="Z124" s="4"/>
       <c r="AA124" s="4"/>
     </row>
-    <row r="125">
-      <c r="A125" s="4"/>
-      <c r="B125" s="4"/>
-      <c r="C125" s="4"/>
-      <c r="D125" s="4"/>
-      <c r="E125" s="4"/>
-      <c r="F125" s="4"/>
-      <c r="G125" s="4"/>
-      <c r="H125" s="4"/>
+    <row r="125" ht="22.5" customHeight="1">
+      <c r="A125" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B125" s="54" t="s">
+        <v>464</v>
+      </c>
+      <c r="C125" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D125" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E125" s="49" t="s">
+        <v>471</v>
+      </c>
+      <c r="F125" s="48" t="s">
+        <v>36</v>
+      </c>
+      <c r="G125" s="49" t="s">
+        <v>226</v>
+      </c>
+      <c r="H125" s="49" t="s">
+        <v>472</v>
+      </c>
       <c r="I125" s="4"/>
       <c r="J125" s="4"/>
       <c r="K125" s="4"/>
@@ -47149,15 +47319,15 @@
       <c r="Z125" s="4"/>
       <c r="AA125" s="4"/>
     </row>
-    <row r="126">
-      <c r="A126" s="4"/>
-      <c r="B126" s="4"/>
-      <c r="C126" s="4"/>
-      <c r="D126" s="4"/>
-      <c r="E126" s="4"/>
-      <c r="F126" s="4"/>
-      <c r="G126" s="4"/>
-      <c r="H126" s="4"/>
+    <row r="126" ht="22.5" customHeight="1">
+      <c r="A126" s="61"/>
+      <c r="B126" s="54"/>
+      <c r="C126" s="48"/>
+      <c r="D126" s="48"/>
+      <c r="E126" s="49"/>
+      <c r="F126" s="50"/>
+      <c r="G126" s="49"/>
+      <c r="H126" s="49"/>
       <c r="I126" s="4"/>
       <c r="J126" s="4"/>
       <c r="K126" s="4"/>
@@ -47178,15 +47348,31 @@
       <c r="Z126" s="4"/>
       <c r="AA126" s="4"/>
     </row>
-    <row r="127">
-      <c r="A127" s="4"/>
-      <c r="B127" s="4"/>
-      <c r="C127" s="4"/>
-      <c r="D127" s="4"/>
-      <c r="E127" s="4"/>
-      <c r="F127" s="4"/>
-      <c r="G127" s="4"/>
-      <c r="H127" s="4"/>
+    <row r="127" ht="22.5" customHeight="1">
+      <c r="A127" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B127" s="54" t="s">
+        <v>473</v>
+      </c>
+      <c r="C127" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D127" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E127" s="49" t="s">
+        <v>474</v>
+      </c>
+      <c r="F127" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="G127" s="49" t="s">
+        <v>239</v>
+      </c>
+      <c r="H127" s="49" t="s">
+        <v>475</v>
+      </c>
       <c r="I127" s="4"/>
       <c r="J127" s="4"/>
       <c r="K127" s="4"/>
@@ -47207,15 +47393,31 @@
       <c r="Z127" s="4"/>
       <c r="AA127" s="4"/>
     </row>
-    <row r="128">
-      <c r="A128" s="4"/>
-      <c r="B128" s="4"/>
-      <c r="C128" s="4"/>
-      <c r="D128" s="4"/>
-      <c r="E128" s="4"/>
-      <c r="F128" s="4"/>
-      <c r="G128" s="4"/>
-      <c r="H128" s="4"/>
+    <row r="128" ht="22.5" customHeight="1">
+      <c r="A128" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B128" s="54" t="s">
+        <v>473</v>
+      </c>
+      <c r="C128" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D128" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E128" s="49" t="s">
+        <v>476</v>
+      </c>
+      <c r="F128" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="G128" s="49" t="s">
+        <v>239</v>
+      </c>
+      <c r="H128" s="49" t="s">
+        <v>477</v>
+      </c>
       <c r="I128" s="4"/>
       <c r="J128" s="4"/>
       <c r="K128" s="4"/>
@@ -47236,15 +47438,31 @@
       <c r="Z128" s="4"/>
       <c r="AA128" s="4"/>
     </row>
-    <row r="129">
-      <c r="A129" s="4"/>
-      <c r="B129" s="4"/>
-      <c r="C129" s="4"/>
-      <c r="D129" s="4"/>
-      <c r="E129" s="4"/>
-      <c r="F129" s="4"/>
-      <c r="G129" s="4"/>
-      <c r="H129" s="4"/>
+    <row r="129" ht="22.5" customHeight="1">
+      <c r="A129" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B129" s="54" t="s">
+        <v>473</v>
+      </c>
+      <c r="C129" s="48" t="s">
+        <v>309</v>
+      </c>
+      <c r="D129" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="E129" s="49" t="s">
+        <v>476</v>
+      </c>
+      <c r="F129" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="G129" s="49" t="s">
+        <v>239</v>
+      </c>
+      <c r="H129" s="49" t="s">
+        <v>478</v>
+      </c>
       <c r="I129" s="4"/>
       <c r="J129" s="4"/>
       <c r="K129" s="4"/>
@@ -47265,15 +47483,15 @@
       <c r="Z129" s="4"/>
       <c r="AA129" s="4"/>
     </row>
-    <row r="130">
-      <c r="A130" s="4"/>
-      <c r="B130" s="4"/>
-      <c r="C130" s="4"/>
-      <c r="D130" s="4"/>
-      <c r="E130" s="4"/>
-      <c r="F130" s="4"/>
-      <c r="G130" s="4"/>
-      <c r="H130" s="4"/>
+    <row r="130" ht="22.5" customHeight="1">
+      <c r="A130" s="50"/>
+      <c r="B130" s="49"/>
+      <c r="C130" s="48"/>
+      <c r="D130" s="48"/>
+      <c r="E130" s="49"/>
+      <c r="F130" s="50"/>
+      <c r="G130" s="49"/>
+      <c r="H130" s="49"/>
       <c r="I130" s="4"/>
       <c r="J130" s="4"/>
       <c r="K130" s="4"/>
@@ -47294,15 +47512,31 @@
       <c r="Z130" s="4"/>
       <c r="AA130" s="4"/>
     </row>
-    <row r="131">
-      <c r="A131" s="4"/>
-      <c r="B131" s="4"/>
-      <c r="C131" s="4"/>
-      <c r="D131" s="4"/>
-      <c r="E131" s="4"/>
-      <c r="F131" s="4"/>
-      <c r="G131" s="4"/>
-      <c r="H131" s="4"/>
+    <row r="131" ht="22.5" customHeight="1">
+      <c r="A131" s="48" t="s">
+        <v>479</v>
+      </c>
+      <c r="B131" s="49" t="s">
+        <v>480</v>
+      </c>
+      <c r="C131" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D131" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E131" s="49" t="s">
+        <v>481</v>
+      </c>
+      <c r="F131" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="G131" s="49" t="s">
+        <v>109</v>
+      </c>
+      <c r="H131" s="49" t="s">
+        <v>482</v>
+      </c>
       <c r="I131" s="4"/>
       <c r="J131" s="4"/>
       <c r="K131" s="4"/>
@@ -47323,15 +47557,31 @@
       <c r="Z131" s="4"/>
       <c r="AA131" s="4"/>
     </row>
-    <row r="132">
-      <c r="A132" s="4"/>
-      <c r="B132" s="4"/>
-      <c r="C132" s="4"/>
-      <c r="D132" s="4"/>
-      <c r="E132" s="4"/>
-      <c r="F132" s="4"/>
-      <c r="G132" s="4"/>
-      <c r="H132" s="4"/>
+    <row r="132" ht="22.5" customHeight="1">
+      <c r="A132" s="48" t="s">
+        <v>479</v>
+      </c>
+      <c r="B132" s="49" t="s">
+        <v>480</v>
+      </c>
+      <c r="C132" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D132" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E132" s="49" t="s">
+        <v>483</v>
+      </c>
+      <c r="F132" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="G132" s="49" t="s">
+        <v>84</v>
+      </c>
+      <c r="H132" s="49" t="s">
+        <v>484</v>
+      </c>
       <c r="I132" s="4"/>
       <c r="J132" s="4"/>
       <c r="K132" s="4"/>
@@ -47352,15 +47602,31 @@
       <c r="Z132" s="4"/>
       <c r="AA132" s="4"/>
     </row>
-    <row r="133">
-      <c r="A133" s="4"/>
-      <c r="B133" s="4"/>
-      <c r="C133" s="4"/>
-      <c r="D133" s="4"/>
-      <c r="E133" s="4"/>
-      <c r="F133" s="4"/>
-      <c r="G133" s="4"/>
-      <c r="H133" s="4"/>
+    <row r="133" ht="22.5" customHeight="1">
+      <c r="A133" s="48" t="s">
+        <v>479</v>
+      </c>
+      <c r="B133" s="49" t="s">
+        <v>485</v>
+      </c>
+      <c r="C133" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D133" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E133" s="49" t="s">
+        <v>486</v>
+      </c>
+      <c r="F133" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="G133" s="49" t="s">
+        <v>100</v>
+      </c>
+      <c r="H133" s="49" t="s">
+        <v>487</v>
+      </c>
       <c r="I133" s="4"/>
       <c r="J133" s="4"/>
       <c r="K133" s="4"/>
@@ -47381,15 +47647,15 @@
       <c r="Z133" s="4"/>
       <c r="AA133" s="4"/>
     </row>
-    <row r="134">
-      <c r="A134" s="4"/>
-      <c r="B134" s="4"/>
-      <c r="C134" s="4"/>
-      <c r="D134" s="4"/>
-      <c r="E134" s="4"/>
-      <c r="F134" s="4"/>
-      <c r="G134" s="4"/>
-      <c r="H134" s="4"/>
+    <row r="134" ht="22.5" customHeight="1">
+      <c r="A134" s="50"/>
+      <c r="B134" s="49"/>
+      <c r="C134" s="48"/>
+      <c r="D134" s="48"/>
+      <c r="E134" s="49"/>
+      <c r="F134" s="50"/>
+      <c r="G134" s="49"/>
+      <c r="H134" s="49"/>
       <c r="I134" s="4"/>
       <c r="J134" s="4"/>
       <c r="K134" s="4"/>
@@ -47410,15 +47676,31 @@
       <c r="Z134" s="4"/>
       <c r="AA134" s="4"/>
     </row>
-    <row r="135">
-      <c r="A135" s="4"/>
-      <c r="B135" s="4"/>
-      <c r="C135" s="4"/>
-      <c r="D135" s="4"/>
-      <c r="E135" s="4"/>
-      <c r="F135" s="4"/>
-      <c r="G135" s="4"/>
-      <c r="H135" s="4"/>
+    <row r="135" ht="22.5" customHeight="1">
+      <c r="A135" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="B135" s="49" t="s">
+        <v>489</v>
+      </c>
+      <c r="C135" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D135" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E135" s="49" t="s">
+        <v>490</v>
+      </c>
+      <c r="F135" s="48" t="s">
+        <v>36</v>
+      </c>
+      <c r="G135" s="49" t="s">
+        <v>226</v>
+      </c>
+      <c r="H135" s="49" t="s">
+        <v>491</v>
+      </c>
       <c r="I135" s="4"/>
       <c r="J135" s="4"/>
       <c r="K135" s="4"/>
@@ -47439,15 +47721,31 @@
       <c r="Z135" s="4"/>
       <c r="AA135" s="4"/>
     </row>
-    <row r="136">
-      <c r="A136" s="4"/>
-      <c r="B136" s="4"/>
-      <c r="C136" s="4"/>
-      <c r="D136" s="4"/>
-      <c r="E136" s="4"/>
-      <c r="F136" s="4"/>
-      <c r="G136" s="4"/>
-      <c r="H136" s="4"/>
+    <row r="136" ht="22.5" customHeight="1">
+      <c r="A136" s="48" t="s">
+        <v>488</v>
+      </c>
+      <c r="B136" s="49" t="s">
+        <v>489</v>
+      </c>
+      <c r="C136" s="48" t="s">
+        <v>306</v>
+      </c>
+      <c r="D136" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E136" s="49" t="s">
+        <v>492</v>
+      </c>
+      <c r="F136" s="48" t="s">
+        <v>36</v>
+      </c>
+      <c r="G136" s="49" t="s">
+        <v>226</v>
+      </c>
+      <c r="H136" s="49" t="s">
+        <v>493</v>
+      </c>
       <c r="I136" s="4"/>
       <c r="J136" s="4"/>
       <c r="K136" s="4"/>
@@ -47468,15 +47766,15 @@
       <c r="Z136" s="4"/>
       <c r="AA136" s="4"/>
     </row>
-    <row r="137">
-      <c r="A137" s="4"/>
-      <c r="B137" s="4"/>
-      <c r="C137" s="4"/>
-      <c r="D137" s="4"/>
-      <c r="E137" s="4"/>
-      <c r="F137" s="4"/>
-      <c r="G137" s="4"/>
-      <c r="H137" s="4"/>
+    <row r="137" ht="22.5" customHeight="1">
+      <c r="A137" s="56"/>
+      <c r="B137" s="57"/>
+      <c r="C137" s="56"/>
+      <c r="D137" s="56"/>
+      <c r="E137" s="57"/>
+      <c r="F137" s="56"/>
+      <c r="G137" s="57"/>
+      <c r="H137" s="57"/>
       <c r="I137" s="4"/>
       <c r="J137" s="4"/>
       <c r="K137" s="4"/>
@@ -73684,47 +73982,18 @@
       <c r="Z1040" s="4"/>
       <c r="AA1040" s="4"/>
     </row>
-    <row r="1041">
-      <c r="A1041" s="4"/>
-      <c r="B1041" s="4"/>
-      <c r="C1041" s="4"/>
-      <c r="D1041" s="4"/>
-      <c r="E1041" s="4"/>
-      <c r="F1041" s="4"/>
-      <c r="G1041" s="4"/>
-      <c r="H1041" s="4"/>
-      <c r="I1041" s="4"/>
-      <c r="J1041" s="4"/>
-      <c r="K1041" s="4"/>
-      <c r="L1041" s="4"/>
-      <c r="M1041" s="4"/>
-      <c r="N1041" s="4"/>
-      <c r="O1041" s="4"/>
-      <c r="P1041" s="4"/>
-      <c r="Q1041" s="4"/>
-      <c r="R1041" s="4"/>
-      <c r="S1041" s="4"/>
-      <c r="T1041" s="4"/>
-      <c r="U1041" s="4"/>
-      <c r="V1041" s="4"/>
-      <c r="W1041" s="4"/>
-      <c r="X1041" s="4"/>
-      <c r="Y1041" s="4"/>
-      <c r="Z1041" s="4"/>
-      <c r="AA1041" s="4"/>
-    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D123">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D137">
       <formula1>"POST,GET,PUT,DELETE,PATCH"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F123">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F137">
       <formula1>"Dilruk Jayasinghe,Kashmika De Silva,Thisal Gannile,Rinusha Nethmini,Indura Amarasekara,Himasha Prabashini,Pahan Gannile"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="A2:A123">
+    <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="A2:A137">
       <formula1>"Authentication,User profile,Support &amp; Inquiries,Customer,Vendor,Admin,Metadata,System &amp; Ops"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C123">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C137">
       <formula1>"Actions,Read,Update,Create,Delete"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>